<commit_message>
Add and update regression scenarios; refresh dashboard run artifacts
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="523">
   <si>
     <t>Run #</t>
   </si>
@@ -830,6 +830,756 @@
   </si>
   <si>
     <t>08/05/2026, 17:04:26</t>
+  </si>
+  <si>
+    <t>CP-MLI-077748131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 08:51:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-077753131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 08:56:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-077754131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 08:59:57</t>
+  </si>
+  <si>
+    <t>CP-MLI-077755131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:02:32</t>
+  </si>
+  <si>
+    <t>CP-NI-077759131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:12:04</t>
+  </si>
+  <si>
+    <t>CP-NI-077760131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:12:53</t>
+  </si>
+  <si>
+    <t>CP-SC-077761131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:13:45</t>
+  </si>
+  <si>
+    <t>CP-SC-077762131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:14:26</t>
+  </si>
+  <si>
+    <t>DA-MLI-077763131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:15:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-077764131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:15:53</t>
+  </si>
+  <si>
+    <t>DA-NI-077765131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:16:44</t>
+  </si>
+  <si>
+    <t>DA-NI-077766131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:17:40</t>
+  </si>
+  <si>
+    <t>DA-SC-077767131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:18:29</t>
+  </si>
+  <si>
+    <t>DA-SC-077768131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:19:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-077769131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:19:56</t>
+  </si>
+  <si>
+    <t>CP-MLI-077770131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:21:15</t>
+  </si>
+  <si>
+    <t>CP-SC-077771131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:22:26</t>
+  </si>
+  <si>
+    <t>DA-MLI-077772131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:23:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-077774131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 09:25:42</t>
+  </si>
+  <si>
+    <t>DA-MLI-077780131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 11:28:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-061533131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 11:35:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-077851131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 14:38:07</t>
+  </si>
+  <si>
+    <t>DA-MLI-077854131</t>
+  </si>
+  <si>
+    <t>TC_REG_014_CNR | Create MTA then start cancel and reissue with return-and-bind at final policy details</t>
+  </si>
+  <si>
+    <t>11/05/2026, 14:46:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-077864131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 15:36:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-077868131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 15:43:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-077870131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 15:51:31</t>
+  </si>
+  <si>
+    <t>DA-MLI-077875131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 15:56:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-077878131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:02:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-077886131</t>
+  </si>
+  <si>
+    <t>TC_REG_035 | CnR then assert Policy Settlement Type is Broker Settled on Details tab</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:23:49</t>
+  </si>
+  <si>
+    <t>DA-MLI-077888131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:28:53</t>
+  </si>
+  <si>
+    <t>CP-MLI-077891131</t>
+  </si>
+  <si>
+    <t>TC_REG_036 | Commercial CnR then assert Policy Settlement Type is Broker Settled on Details tab</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:35:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-077895131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:49:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-077900131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 16:55:11</t>
+  </si>
+  <si>
+    <t>CP-MLI-061550131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 18:37:46</t>
+  </si>
+  <si>
+    <t>CP-MLI-061552131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 18:39:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-061558131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 18:52:37</t>
+  </si>
+  <si>
+    <t>CP-NI-061565131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:18:27</t>
+  </si>
+  <si>
+    <t>CP-NI-061566131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:19:26</t>
+  </si>
+  <si>
+    <t>CP-SC-061567131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:20:29</t>
+  </si>
+  <si>
+    <t>CP-SC-061568131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:21:57</t>
+  </si>
+  <si>
+    <t>DA-MLI-061569131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:22:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-061570131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:23:47</t>
+  </si>
+  <si>
+    <t>DA-NI-061571131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:25:02</t>
+  </si>
+  <si>
+    <t>DA-NI-061572131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:25:52</t>
+  </si>
+  <si>
+    <t>DA-SC-061573131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:26:50</t>
+  </si>
+  <si>
+    <t>DA-SC-061574131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:27:54</t>
+  </si>
+  <si>
+    <t>DA-MLI-061575131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:28:50</t>
+  </si>
+  <si>
+    <t>CP-MLI-061576131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:30:16</t>
+  </si>
+  <si>
+    <t>CP-SC-061577131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:31:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-061578131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:33:03</t>
+  </si>
+  <si>
+    <t>DA-MLI-061580131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 19:35:54</t>
+  </si>
+  <si>
+    <t>CP-MLI-061587131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 20:01:39</t>
+  </si>
+  <si>
+    <t>CP-MLI-061590131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 20:02:40</t>
+  </si>
+  <si>
+    <t>DA-MLI-061593131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 20:05:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-061595131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 20:07:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-061597131</t>
+  </si>
+  <si>
+    <t>11/05/2026, 20:17:25</t>
+  </si>
+  <si>
+    <t>CP-MLI-061626132</t>
+  </si>
+  <si>
+    <t>TC_REG_036 | Commercial CnR then assert Policy Settlement Type is Broker Settled on Details tab (Commercial)</t>
+  </si>
+  <si>
+    <t>12/05/2026, 14:52:25</t>
+  </si>
+  <si>
+    <t>CP-MLI-061653132</t>
+  </si>
+  <si>
+    <t>TC_REG_037 | Commercial CnR then assert Policy Settlement Type is Over Settled on Details tab</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:02:10</t>
+  </si>
+  <si>
+    <t>CP-MLI-061683132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:35:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-061685132</t>
+  </si>
+  <si>
+    <t>TC_REG_038 | Create MTA then Change Stage to Declined and assert stage</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:46:17</t>
+  </si>
+  <si>
+    <t>DA-MLI-061686132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:48:49</t>
+  </si>
+  <si>
+    <t>DA-MLI-061687132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:51:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-061689132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:55:23</t>
+  </si>
+  <si>
+    <t>CP-MLI-061693132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 15:59:38</t>
+  </si>
+  <si>
+    <t>CP-MLI-061695132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:01:26</t>
+  </si>
+  <si>
+    <t>DA-MLI-061700132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:07:38</t>
+  </si>
+  <si>
+    <t>DA-MLI-061701132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:10:38</t>
+  </si>
+  <si>
+    <t>CP-NI-061702132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:13:39</t>
+  </si>
+  <si>
+    <t>CP-NI-061703132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:14:40</t>
+  </si>
+  <si>
+    <t>CP-SC-061704132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:15:48</t>
+  </si>
+  <si>
+    <t>CP-SC-061705132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:16:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-061706132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:17:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-061707132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:18:51</t>
+  </si>
+  <si>
+    <t>DA-NI-061708132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:20:01</t>
+  </si>
+  <si>
+    <t>DA-NI-061709132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:21:02</t>
+  </si>
+  <si>
+    <t>DA-SC-061710132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:22:00</t>
+  </si>
+  <si>
+    <t>DA-SC-061711132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:23:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-061712132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:24:05</t>
+  </si>
+  <si>
+    <t>CP-MLI-061713132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:25:26</t>
+  </si>
+  <si>
+    <t>DA-MLI-061715132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:28:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-061717132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:32:08</t>
+  </si>
+  <si>
+    <t>CP-NI-061719132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:37:27</t>
+  </si>
+  <si>
+    <t>CP-NI-061720132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:38:39</t>
+  </si>
+  <si>
+    <t>CP-SC-061721132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:39:50</t>
+  </si>
+  <si>
+    <t>CP-SC-061722132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:40:49</t>
+  </si>
+  <si>
+    <t>DA-MLI-061723132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:41:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-061724132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:42:48</t>
+  </si>
+  <si>
+    <t>DA-NI-061725132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:43:44</t>
+  </si>
+  <si>
+    <t>DA-NI-061726132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:44:49</t>
+  </si>
+  <si>
+    <t>DA-SC-061727132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:45:45</t>
+  </si>
+  <si>
+    <t>DA-SC-061728132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:46:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-061729132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:47:37</t>
+  </si>
+  <si>
+    <t>CP-MLI-061730132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:49:01</t>
+  </si>
+  <si>
+    <t>CP-SC-061731132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:50:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-061732132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:51:52</t>
+  </si>
+  <si>
+    <t>DA-MLI-061734132</t>
+  </si>
+  <si>
+    <t>12/05/2026, 16:55:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-079933133</t>
+  </si>
+  <si>
+    <t>TC_REG_040 | Create claim then create MTA from Risk ID and assert claim warning text</t>
+  </si>
+  <si>
+    <t>13/05/2026, 12:32:52</t>
+  </si>
+  <si>
+    <t>DA-MLI-079935133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 12:39:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-079936133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 12:43:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-079937133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 12:53:29</t>
+  </si>
+  <si>
+    <t>DA-MLI-079939133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 12:57:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-079940133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 13:02:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-079942133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 13:05:07</t>
+  </si>
+  <si>
+    <t>DA-MLI-079943133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 13:08:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-062603133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 13:13:38</t>
+  </si>
+  <si>
+    <t>CP-MLI-537179133</t>
+  </si>
+  <si>
+    <t>UAT2</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:30:44</t>
+  </si>
+  <si>
+    <t>CP-MLI-537181133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:32:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-537201133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:35:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-537202133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:37:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-537213133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:39:53</t>
+  </si>
+  <si>
+    <t>CP-MLI-537250133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:47:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-537261133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:48:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-537264133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 14:50:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-079955133</t>
+  </si>
+  <si>
+    <t>TC_REG_041 | Assert Debit Note premium before and after MTA from Source Submission</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:03:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-079956133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:06:52</t>
+  </si>
+  <si>
+    <t>DA-MLI-079957133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:11:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-079958133</t>
+  </si>
+  <si>
+    <t>TC_REG_041 | Open Debit Note before and after MTA from Source Submission</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:14:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-079959133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:18:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-079960133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:23:23</t>
+  </si>
+  <si>
+    <t>DA-MLI-062604133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:27:19</t>
   </si>
 </sst>
 </file>
@@ -1263,7 +2013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F234"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3554,6 +4304,2406 @@
         <v>272</v>
       </c>
     </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="4">
+        <v>114</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C115" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F115" s="5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="2">
+        <v>115</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="4">
+        <v>116</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C117" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E117" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F117" s="5" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="2">
+        <v>117</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="4">
+        <v>118</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E119" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F119" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="2">
+        <v>119</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" s="4">
+        <v>120</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="2">
+        <v>121</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="4">
+        <v>122</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F123" s="5" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="2">
+        <v>123</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" s="4">
+        <v>124</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F125" s="5" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" s="2">
+        <v>125</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" s="4">
+        <v>126</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F127" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" s="2">
+        <v>127</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" s="4">
+        <v>128</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" s="2">
+        <v>129</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="4">
+        <v>130</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" s="2">
+        <v>131</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="4">
+        <v>132</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E133" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F133" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="2">
+        <v>133</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="4">
+        <v>134</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E135" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F135" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="2">
+        <v>135</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" s="4">
+        <v>136</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F137" s="5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" s="2">
+        <v>137</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" s="4">
+        <v>138</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" s="2">
+        <v>139</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" s="4">
+        <v>140</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" s="2">
+        <v>141</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" s="4">
+        <v>142</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E143" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F143" s="5" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" s="2">
+        <v>143</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" s="4">
+        <v>144</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E145" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F145" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" s="2">
+        <v>145</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" s="4">
+        <v>146</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="C147" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E147" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F147" s="5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" s="2">
+        <v>147</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" s="4">
+        <v>148</v>
+      </c>
+      <c r="B149" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C149" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E149" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F149" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" s="2">
+        <v>149</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" s="4">
+        <v>150</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C151" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D151" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E151" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F151" s="5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" s="2">
+        <v>151</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" s="4">
+        <v>152</v>
+      </c>
+      <c r="B153" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C153" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E153" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F153" s="5" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" s="2">
+        <v>153</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155" s="4">
+        <v>154</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156" s="2">
+        <v>155</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157" s="4">
+        <v>156</v>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="C157" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E157" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158" s="2">
+        <v>157</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D158" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159" s="4">
+        <v>158</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E159" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160" s="2">
+        <v>159</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161" s="4">
+        <v>160</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="C161" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E161" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F161" s="5" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162" s="2">
+        <v>161</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E162" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163" s="4">
+        <v>162</v>
+      </c>
+      <c r="B163" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D163" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E163" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F163" s="5" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164" s="2">
+        <v>163</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E164" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165" s="4">
+        <v>164</v>
+      </c>
+      <c r="B165" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="C165" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E165" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F165" s="5" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166" s="2">
+        <v>165</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E166" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167" s="4">
+        <v>166</v>
+      </c>
+      <c r="B167" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="C167" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E167" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F167" s="5" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" s="2">
+        <v>167</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" s="4">
+        <v>168</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E169" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F169" s="5" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" s="2">
+        <v>169</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D170" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E170" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" s="4">
+        <v>170</v>
+      </c>
+      <c r="B171" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="C171" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D171" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E171" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F171" s="5" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" s="2">
+        <v>171</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C172" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E172" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" s="4">
+        <v>172</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D173" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E173" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F173" s="5" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" s="2">
+        <v>173</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C174" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D174" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E174" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F174" s="3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" s="4">
+        <v>174</v>
+      </c>
+      <c r="B175" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="C175" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="D175" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E175" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F175" s="5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" s="2">
+        <v>175</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E176" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F176" s="3" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" s="4">
+        <v>176</v>
+      </c>
+      <c r="B177" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="D177" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E177" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F177" s="5" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="2">
+        <v>177</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D178" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E178" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F178" s="3" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="4">
+        <v>178</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E179" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F179" s="5" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="2">
+        <v>179</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E180" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="4">
+        <v>180</v>
+      </c>
+      <c r="B181" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="C181" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D181" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E181" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F181" s="5" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" s="2">
+        <v>181</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D182" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E182" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F182" s="3" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" s="4">
+        <v>182</v>
+      </c>
+      <c r="B183" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="C183" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D183" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E183" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F183" s="5" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" s="2">
+        <v>183</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D184" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E184" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F184" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" s="4">
+        <v>184</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="C185" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D185" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E185" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F185" s="5" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" s="2">
+        <v>185</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D186" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E186" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F186" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" s="4">
+        <v>186</v>
+      </c>
+      <c r="B187" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="C187" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D187" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E187" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F187" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" s="2">
+        <v>187</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D188" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E188" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F188" s="3" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" s="4">
+        <v>188</v>
+      </c>
+      <c r="B189" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="C189" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E189" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F189" s="5" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" s="2">
+        <v>189</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D190" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E190" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F190" s="3" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" s="4">
+        <v>190</v>
+      </c>
+      <c r="B191" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="C191" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E191" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F191" s="5" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" s="2">
+        <v>191</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="C192" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D192" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E192" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F192" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" s="4">
+        <v>192</v>
+      </c>
+      <c r="B193" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="C193" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D193" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E193" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F193" s="5" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" s="2">
+        <v>193</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" s="4">
+        <v>194</v>
+      </c>
+      <c r="B195" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="C195" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E195" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F195" s="5" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A196" s="2">
+        <v>195</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E196" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F196" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A197" s="4">
+        <v>196</v>
+      </c>
+      <c r="B197" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="C197" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E197" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F197" s="5" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A198" s="2">
+        <v>197</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F198" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A199" s="4">
+        <v>198</v>
+      </c>
+      <c r="B199" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C199" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E199" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F199" s="5" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A200" s="2">
+        <v>199</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E200" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F200" s="3" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A201" s="4">
+        <v>200</v>
+      </c>
+      <c r="B201" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="C201" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D201" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E201" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F201" s="5" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A202" s="2">
+        <v>201</v>
+      </c>
+      <c r="B202" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E202" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F202" s="3" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" s="4">
+        <v>202</v>
+      </c>
+      <c r="B203" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="C203" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D203" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E203" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F203" s="5" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" s="2">
+        <v>203</v>
+      </c>
+      <c r="B204" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D204" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E204" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F204" s="3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" s="4">
+        <v>204</v>
+      </c>
+      <c r="B205" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="C205" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D205" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E205" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F205" s="5" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" s="2">
+        <v>205</v>
+      </c>
+      <c r="B206" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D206" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E206" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F206" s="3" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" s="4">
+        <v>206</v>
+      </c>
+      <c r="B207" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="C207" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D207" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E207" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F207" s="5" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" s="2">
+        <v>207</v>
+      </c>
+      <c r="B208" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D208" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F208" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" s="4">
+        <v>208</v>
+      </c>
+      <c r="B209" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="C209" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D209" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E209" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F209" s="5" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A210" s="2">
+        <v>209</v>
+      </c>
+      <c r="B210" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D210" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E210" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F210" s="3" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A211" s="4">
+        <v>210</v>
+      </c>
+      <c r="B211" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="C211" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D211" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E211" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F211" s="5" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" s="2">
+        <v>211</v>
+      </c>
+      <c r="B212" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E212" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A213" s="4">
+        <v>212</v>
+      </c>
+      <c r="B213" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C213" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D213" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E213" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F213" s="5" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A214" s="2">
+        <v>213</v>
+      </c>
+      <c r="B214" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E214" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F214" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A215" s="4">
+        <v>214</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="C215" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D215" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E215" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F215" s="5" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A216" s="2">
+        <v>215</v>
+      </c>
+      <c r="B216" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E216" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F216" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A217" s="4">
+        <v>216</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D217" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E217" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F217" s="5" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A218" s="2">
+        <v>217</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D218" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E218" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A219" s="4">
+        <v>218</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="C219" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D219" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E219" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F219" s="5" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A220" s="2">
+        <v>219</v>
+      </c>
+      <c r="B220" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E220" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A221" s="4">
+        <v>220</v>
+      </c>
+      <c r="B221" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="C221" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E221" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F221" s="5" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A222" s="2">
+        <v>221</v>
+      </c>
+      <c r="B222" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E222" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A223" s="4">
+        <v>222</v>
+      </c>
+      <c r="B223" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="C223" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D223" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E223" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F223" s="5" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A224" s="2">
+        <v>223</v>
+      </c>
+      <c r="B224" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E224" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A225" s="4">
+        <v>224</v>
+      </c>
+      <c r="B225" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="C225" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D225" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E225" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F225" s="5" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A226" s="2">
+        <v>225</v>
+      </c>
+      <c r="B226" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E226" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F226" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A227" s="4">
+        <v>226</v>
+      </c>
+      <c r="B227" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D227" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E227" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F227" s="5" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A228" s="2">
+        <v>227</v>
+      </c>
+      <c r="B228" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E228" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F228" s="3" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A229" s="4">
+        <v>228</v>
+      </c>
+      <c r="B229" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="C229" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D229" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E229" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F229" s="5" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A230" s="2">
+        <v>229</v>
+      </c>
+      <c r="B230" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E230" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F230" s="3" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A231" s="4">
+        <v>230</v>
+      </c>
+      <c r="B231" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="C231" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="D231" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E231" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F231" s="5" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A232" s="2">
+        <v>231</v>
+      </c>
+      <c r="B232" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E232" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F232" s="3" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A233" s="4">
+        <v>232</v>
+      </c>
+      <c r="B233" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="C233" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D233" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E233" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F233" s="5" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A234" s="2">
+        <v>233</v>
+      </c>
+      <c r="B234" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E234" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F234" s="3" t="s">
+        <v>522</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Add MTA descriptions and post-bind Risk ID assertions across tests
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="817">
   <si>
     <t>Run #</t>
   </si>
@@ -1580,6 +1580,888 @@
   </si>
   <si>
     <t>13/05/2026, 15:27:19</t>
+  </si>
+  <si>
+    <t>DA-MLI-537284133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:54:39</t>
+  </si>
+  <si>
+    <t>DA-MLI-537285133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:56:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-080082134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 11:49:36</t>
+  </si>
+  <si>
+    <t>CP-MLI-062655134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 13:23:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-080091134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 13:48:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-080095134</t>
+  </si>
+  <si>
+    <t>TC_REG_042 | Cancel and reissue date today then MTA effective date cannot be yesterday</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:02:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-080099134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:07:56</t>
+  </si>
+  <si>
+    <t>DA-MLI-080102134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:14:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-080105134</t>
+  </si>
+  <si>
+    <t>TC_REG_043 | Create MTA then Cancel and Reissue then Create MTA</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:28:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-080112134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:40:30</t>
+  </si>
+  <si>
+    <t>DA-MLI-537294134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:52:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-537296134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:55:48</t>
+  </si>
+  <si>
+    <t>CP-MLI-062657134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:17:43</t>
+  </si>
+  <si>
+    <t>CP-MLI-062659134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:19:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-062679134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:24:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-062688134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:27:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-062705134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:30:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-080120134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:43:05</t>
+  </si>
+  <si>
+    <t>CP-NI-080127134</t>
+  </si>
+  <si>
+    <t>DT-MLIS-DF25.5.0 | CR-237340 |TC_34_S6_Verify Cancellation premiums are applied to the appropriate intermediary when user change the Intermediary Legal Entity on MTA _NB&gt;CRN&gt;MTA_Cancel the Policy Mid-term_NI commercial_Broker portal</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:19:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080129134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:23:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080132134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:28:52</t>
+  </si>
+  <si>
+    <t>CP-NI-080495138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:32:40</t>
+  </si>
+  <si>
+    <t>CP-NI-080497138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:37:13</t>
+  </si>
+  <si>
+    <t>CP-NI-080499138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:41:41</t>
+  </si>
+  <si>
+    <t>CP-NI-080501138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:45:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080503138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:49:18</t>
+  </si>
+  <si>
+    <t>CP-NI-080506138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:53:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080510138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:02:42</t>
+  </si>
+  <si>
+    <t>CP-NI-080513138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:08:11</t>
+  </si>
+  <si>
+    <t>CP-NI-080516138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:12:55</t>
+  </si>
+  <si>
+    <t>CP-NI-080517138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:14:47</t>
+  </si>
+  <si>
+    <t>CP-NI-080520138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:21:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080523138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:26:08</t>
+  </si>
+  <si>
+    <t>CP-NI-080526138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:31:55</t>
+  </si>
+  <si>
+    <t>CP-NI-080528138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:37:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080532138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:46:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080535138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:53:45</t>
+  </si>
+  <si>
+    <t>CP-NI-080538138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:02:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080541138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:09:12</t>
+  </si>
+  <si>
+    <t>CP-NI-080544138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:15:18</t>
+  </si>
+  <si>
+    <t>CP-NI-080547138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:20:19</t>
+  </si>
+  <si>
+    <t>CP-NI-080550138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:27:05</t>
+  </si>
+  <si>
+    <t>CP-NI-080553138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:32:16</t>
+  </si>
+  <si>
+    <t>CP-NI-080555138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:35:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080558138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:41:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080561138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:51:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080564138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:00:13</t>
+  </si>
+  <si>
+    <t>CP-NI-062979138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:04:14</t>
+  </si>
+  <si>
+    <t>CP-NI-080567138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:17:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080570138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:22:21</t>
+  </si>
+  <si>
+    <t>CP-NI-080572138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:24:42</t>
+  </si>
+  <si>
+    <t>CP-NI-080575138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:29:27</t>
+  </si>
+  <si>
+    <t>CP-NI-080577138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:32:10</t>
+  </si>
+  <si>
+    <t>CP-NI-080580138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:38:36</t>
+  </si>
+  <si>
+    <t>CP-NI-080583138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:43:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080586138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:48:56</t>
+  </si>
+  <si>
+    <t>CP-NI-080589138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:55:02</t>
+  </si>
+  <si>
+    <t>CP-NI-080593138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:02:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080596138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:08:40</t>
+  </si>
+  <si>
+    <t>CP-NI-080599138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:14:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080602138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:21:46</t>
+  </si>
+  <si>
+    <t>CP-NI-080605138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:27:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080606138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:29:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080608138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:33:04</t>
+  </si>
+  <si>
+    <t>DA-MLI-080624138</t>
+  </si>
+  <si>
+    <t>TC_REG_045 | Source Submission -&gt; Change of Limit of Indemnity updates Limit of Indemnity after refresh</t>
+  </si>
+  <si>
+    <t>18/05/2026, 13:45:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-080626138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 13:51:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080628138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:00:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080672138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:11:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080717138</t>
+  </si>
+  <si>
+    <t>TC_REG_045 | Clear MTA flow on a live policy</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:25:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-080719138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:27:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-080722138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:29:04</t>
+  </si>
+  <si>
+    <t>DA-MLI-080726138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:33:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-080728138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:35:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-080729138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:38:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-080732138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:43:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-080735138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:46:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-080737138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:51:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080738138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:52:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080741138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:55:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080743138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:59:36</t>
+  </si>
+  <si>
+    <t>DA-MLI-080744138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:02:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-080745138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:04:44</t>
+  </si>
+  <si>
+    <t>DA-MLI-080747138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:09:36</t>
+  </si>
+  <si>
+    <t>DA-MLI-080750138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:14:18</t>
+  </si>
+  <si>
+    <t>DA-MLI-080753138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:20:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-080755138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:23:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-080759138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:29:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-080769138</t>
+  </si>
+  <si>
+    <t>TC_REG_046 | Create MTA without bind, assert Insurance Policies (0) and Quotes (1), open Quote</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:17:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-080770138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:21:29</t>
+  </si>
+  <si>
+    <t>DA-MLI-080773138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:25:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080776138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:35:28</t>
+  </si>
+  <si>
+    <t>CP-NI-080780138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:42:16</t>
+  </si>
+  <si>
+    <t>CP-NI-080783138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:48:31</t>
+  </si>
+  <si>
+    <t>CP-NI-080787138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:54:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080789138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:57:11</t>
+  </si>
+  <si>
+    <t>CP-NI-080794138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:09:08</t>
+  </si>
+  <si>
+    <t>CP-NI-080798138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:15:09</t>
+  </si>
+  <si>
+    <t>CP-NI-063006138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:59:05</t>
+  </si>
+  <si>
+    <t>CP-NI-063005138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:00:36</t>
+  </si>
+  <si>
+    <t>CP-NI-080817138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:02:27</t>
+  </si>
+  <si>
+    <t>CP-NI-080823138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:07:26</t>
+  </si>
+  <si>
+    <t>CP-NI-080828138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:15:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080835138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:26:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080956139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:10:46</t>
+  </si>
+  <si>
+    <t>CP-NI-080961139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:19:59</t>
+  </si>
+  <si>
+    <t>CP-NI-080969139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:32:28</t>
+  </si>
+  <si>
+    <t>CP-NI-080971139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:35:48</t>
+  </si>
+  <si>
+    <t>CP-NI-080973139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:38:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080974139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:40:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-063700140</t>
+  </si>
+  <si>
+    <t>TC_BDX_005_NB_MTA | Create NB-MTA (Mid-Term Adjustment) on a live policy</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:04:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-081093140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:06:43</t>
+  </si>
+  <si>
+    <t>DA-MLI-081094140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:10:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-081095140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:10:24</t>
+  </si>
+  <si>
+    <t>DA-MLI-081098140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:13:48</t>
+  </si>
+  <si>
+    <t>CP-MLI-081106140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:44:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-063836140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:50:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063843140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:55:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-063847140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:57:13</t>
+  </si>
+  <si>
+    <t>CP-MLI-063851140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:59:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-063852140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:59:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-081125140</t>
+  </si>
+  <si>
+    <t>TC_REG_047 | Save at quotes, verify SF related counts, resume and issue policy</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:37:39</t>
+  </si>
+  <si>
+    <t>DA-MLI-081127140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:46:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-081129140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:55:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-081130140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:01:19</t>
+  </si>
+  <si>
+    <t>DA-MLI-081133140</t>
+  </si>
+  <si>
+    <t>TC_REG_048 | NB-MTA validate Edit Terms Discount + Update Premium fallback and complete bind</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:43:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-081134140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:50:38</t>
+  </si>
+  <si>
+    <t>DA-MLI-081136140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:54:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-081138140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:00:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-081141140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:11:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-081143140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:21:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-081148140</t>
+  </si>
+  <si>
+    <t>TC_REG_049 | Create NB then update discount on Quotes tab and continue quote in Salesforce</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:46:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-063952140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:50:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063954140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:53:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-063955140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:54:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-063956140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:59:42</t>
+  </si>
+  <si>
+    <t>DA-MLI-063967140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:40:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063971140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:53:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-063974140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:59:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-063977140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 19:09:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-081322141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 15:55:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-081332141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 16:00:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-081334141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 16:02:27</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F234"/>
+  <dimension ref="A1:F376"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -6704,6 +7586,2846 @@
         <v>522</v>
       </c>
     </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" s="4">
+        <v>234</v>
+      </c>
+      <c r="B235" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="C235" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D235" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E235" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F235" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" s="2">
+        <v>235</v>
+      </c>
+      <c r="B236" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E236" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F236" s="3" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" s="4">
+        <v>236</v>
+      </c>
+      <c r="B237" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="C237" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D237" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E237" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F237" s="5" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" s="2">
+        <v>237</v>
+      </c>
+      <c r="B238" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E238" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F238" s="3" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" s="4">
+        <v>238</v>
+      </c>
+      <c r="B239" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="C239" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E239" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F239" s="5" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" s="2">
+        <v>239</v>
+      </c>
+      <c r="B240" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D240" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E240" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F240" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A241" s="4">
+        <v>240</v>
+      </c>
+      <c r="B241" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="C241" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="D241" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E241" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F241" s="5" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A242" s="2">
+        <v>241</v>
+      </c>
+      <c r="B242" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E242" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F242" s="3" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A243" s="4">
+        <v>242</v>
+      </c>
+      <c r="B243" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="C243" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="D243" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E243" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F243" s="5" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A244" s="2">
+        <v>243</v>
+      </c>
+      <c r="B244" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E244" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F244" s="3" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A245" s="4">
+        <v>244</v>
+      </c>
+      <c r="B245" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="C245" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D245" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E245" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A246" s="2">
+        <v>245</v>
+      </c>
+      <c r="B246" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E246" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A247" s="4">
+        <v>246</v>
+      </c>
+      <c r="B247" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C247" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E247" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F247" s="5" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A248" s="2">
+        <v>247</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E248" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F248" s="3" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A249" s="4">
+        <v>248</v>
+      </c>
+      <c r="B249" s="5" t="s">
+        <v>553</v>
+      </c>
+      <c r="C249" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E249" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F249" s="5" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A250" s="2">
+        <v>249</v>
+      </c>
+      <c r="B250" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E250" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F250" s="3" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A251" s="4">
+        <v>250</v>
+      </c>
+      <c r="B251" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="C251" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E251" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F251" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A252" s="2">
+        <v>251</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E252" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F252" s="3" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A253" s="4">
+        <v>252</v>
+      </c>
+      <c r="B253" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="C253" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E253" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F253" s="5" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A254" s="2">
+        <v>253</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E254" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F254" s="3" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A255" s="4">
+        <v>254</v>
+      </c>
+      <c r="B255" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="C255" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E255" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F255" s="5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A256" s="2">
+        <v>255</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E256" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F256" s="3" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A257" s="4">
+        <v>256</v>
+      </c>
+      <c r="B257" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="C257" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E257" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F257" s="5" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A258" s="2">
+        <v>257</v>
+      </c>
+      <c r="B258" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D258" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E258" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F258" s="3" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A259" s="4">
+        <v>258</v>
+      </c>
+      <c r="B259" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="C259" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D259" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E259" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F259" s="5" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A260" s="2">
+        <v>259</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F260" s="3" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A261" s="4">
+        <v>260</v>
+      </c>
+      <c r="B261" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="C261" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E261" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F261" s="5" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A262" s="2">
+        <v>261</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F262" s="3" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A263" s="4">
+        <v>262</v>
+      </c>
+      <c r="B263" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="C263" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D263" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E263" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F263" s="5" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A264" s="2">
+        <v>263</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F264" s="3" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A265" s="4">
+        <v>264</v>
+      </c>
+      <c r="B265" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="C265" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D265" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E265" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F265" s="5" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A266" s="2">
+        <v>265</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D266" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F266" s="3" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A267" s="4">
+        <v>266</v>
+      </c>
+      <c r="B267" s="5" t="s">
+        <v>590</v>
+      </c>
+      <c r="C267" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E267" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A268" s="2">
+        <v>267</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D268" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E268" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F268" s="3" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A269" s="4">
+        <v>268</v>
+      </c>
+      <c r="B269" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="C269" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D269" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E269" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F269" s="5" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A270" s="2">
+        <v>269</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D270" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E270" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F270" s="3" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A271" s="4">
+        <v>270</v>
+      </c>
+      <c r="B271" s="5" t="s">
+        <v>598</v>
+      </c>
+      <c r="C271" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E271" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F271" s="5" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A272" s="2">
+        <v>271</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D272" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E272" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F272" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A273" s="4">
+        <v>272</v>
+      </c>
+      <c r="B273" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="C273" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E273" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F273" s="5" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A274" s="2">
+        <v>273</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D274" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A275" s="4">
+        <v>274</v>
+      </c>
+      <c r="B275" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="C275" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E275" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A276" s="2">
+        <v>275</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E276" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F276" s="3" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A277" s="4">
+        <v>276</v>
+      </c>
+      <c r="B277" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="C277" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D277" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E277" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F277" s="5" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A278" s="2">
+        <v>277</v>
+      </c>
+      <c r="B278" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D278" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E278" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A279" s="4">
+        <v>278</v>
+      </c>
+      <c r="B279" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="C279" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D279" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E279" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F279" s="5" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A280" s="2">
+        <v>279</v>
+      </c>
+      <c r="B280" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A281" s="4">
+        <v>280</v>
+      </c>
+      <c r="B281" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="C281" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E281" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A282" s="2">
+        <v>281</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D282" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E282" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F282" s="3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A283" s="4">
+        <v>282</v>
+      </c>
+      <c r="B283" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="C283" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E283" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A284" s="2">
+        <v>283</v>
+      </c>
+      <c r="B284" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D284" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E284" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F284" s="3" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A285" s="4">
+        <v>284</v>
+      </c>
+      <c r="B285" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="C285" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E285" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A286" s="2">
+        <v>285</v>
+      </c>
+      <c r="B286" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F286" s="3" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A287" s="4">
+        <v>286</v>
+      </c>
+      <c r="B287" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="C287" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E287" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F287" s="5" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A288" s="2">
+        <v>287</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F288" s="3" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A289" s="4">
+        <v>288</v>
+      </c>
+      <c r="B289" s="5" t="s">
+        <v>634</v>
+      </c>
+      <c r="C289" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D289" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E289" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F289" s="5" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A290" s="2">
+        <v>289</v>
+      </c>
+      <c r="B290" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F290" s="3" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A291" s="4">
+        <v>290</v>
+      </c>
+      <c r="B291" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="C291" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E291" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A292" s="2">
+        <v>291</v>
+      </c>
+      <c r="B292" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A293" s="4">
+        <v>292</v>
+      </c>
+      <c r="B293" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="C293" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E293" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F293" s="5" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A294" s="2">
+        <v>293</v>
+      </c>
+      <c r="B294" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A295" s="4">
+        <v>294</v>
+      </c>
+      <c r="B295" s="5" t="s">
+        <v>646</v>
+      </c>
+      <c r="C295" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E295" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A296" s="2">
+        <v>295</v>
+      </c>
+      <c r="B296" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F296" s="3" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A297" s="4">
+        <v>296</v>
+      </c>
+      <c r="B297" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="C297" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E297" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A298" s="2">
+        <v>297</v>
+      </c>
+      <c r="B298" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F298" s="3" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A299" s="4">
+        <v>298</v>
+      </c>
+      <c r="B299" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="C299" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E299" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A300" s="2">
+        <v>299</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A301" s="4">
+        <v>300</v>
+      </c>
+      <c r="B301" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="C301" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E301" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F301" s="5" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A302" s="2">
+        <v>301</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A303" s="4">
+        <v>302</v>
+      </c>
+      <c r="B303" s="5" t="s">
+        <v>663</v>
+      </c>
+      <c r="C303" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E303" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F303" s="5" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A304" s="2">
+        <v>303</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A305" s="4">
+        <v>304</v>
+      </c>
+      <c r="B305" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="C305" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D305" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E305" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F305" s="5" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A306" s="2">
+        <v>305</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F306" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A307" s="4">
+        <v>306</v>
+      </c>
+      <c r="B307" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="C307" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E307" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F307" s="5" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A308" s="2">
+        <v>307</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>674</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F308" s="3" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A309" s="4">
+        <v>308</v>
+      </c>
+      <c r="B309" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="C309" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E309" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F309" s="5" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A310" s="2">
+        <v>309</v>
+      </c>
+      <c r="B310" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F310" s="3" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A311" s="4">
+        <v>310</v>
+      </c>
+      <c r="B311" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="C311" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D311" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E311" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F311" s="5" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A312" s="2">
+        <v>311</v>
+      </c>
+      <c r="B312" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F312" s="3" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A313" s="4">
+        <v>312</v>
+      </c>
+      <c r="B313" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="C313" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D313" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E313" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F313" s="5" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A314" s="2">
+        <v>313</v>
+      </c>
+      <c r="B314" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E314" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F314" s="3" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A315" s="4">
+        <v>314</v>
+      </c>
+      <c r="B315" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="C315" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D315" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E315" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F315" s="5" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A316" s="2">
+        <v>315</v>
+      </c>
+      <c r="B316" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E316" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F316" s="3" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A317" s="4">
+        <v>316</v>
+      </c>
+      <c r="B317" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="C317" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D317" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E317" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F317" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A318" s="2">
+        <v>317</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E318" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F318" s="3" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A319" s="4">
+        <v>318</v>
+      </c>
+      <c r="B319" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="C319" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D319" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E319" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F319" s="5" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A320" s="2">
+        <v>319</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E320" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F320" s="3" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321" s="4">
+        <v>320</v>
+      </c>
+      <c r="B321" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="C321" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D321" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E321" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F321" s="5" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A322" s="2">
+        <v>321</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="C322" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D322" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E322" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F322" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A323" s="4">
+        <v>322</v>
+      </c>
+      <c r="B323" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="C323" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="D323" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E323" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F323" s="5" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A324" s="2">
+        <v>323</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="C324" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D324" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E324" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F324" s="3" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A325" s="4">
+        <v>324</v>
+      </c>
+      <c r="B325" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="C325" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D325" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E325" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F325" s="5" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A326" s="2">
+        <v>325</v>
+      </c>
+      <c r="B326" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="C326" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D326" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E326" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F326" s="3" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A327" s="4">
+        <v>326</v>
+      </c>
+      <c r="B327" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="C327" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D327" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E327" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F327" s="5" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A328" s="2">
+        <v>327</v>
+      </c>
+      <c r="B328" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="C328" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D328" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E328" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F328" s="3" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A329" s="4">
+        <v>328</v>
+      </c>
+      <c r="B329" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="C329" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D329" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E329" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F329" s="5" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A330" s="2">
+        <v>329</v>
+      </c>
+      <c r="B330" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="C330" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D330" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E330" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F330" s="3" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A331" s="4">
+        <v>330</v>
+      </c>
+      <c r="B331" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="C331" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D331" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E331" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F331" s="5" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A332" s="2">
+        <v>331</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="C332" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D332" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E332" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F332" s="3" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A333" s="4">
+        <v>332</v>
+      </c>
+      <c r="B333" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="C333" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D333" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E333" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F333" s="5" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A334" s="2">
+        <v>333</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>727</v>
+      </c>
+      <c r="C334" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D334" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E334" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F334" s="3" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A335" s="4">
+        <v>334</v>
+      </c>
+      <c r="B335" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="C335" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D335" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E335" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F335" s="5" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A336" s="2">
+        <v>335</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="C336" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D336" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E336" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F336" s="3" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A337" s="4">
+        <v>336</v>
+      </c>
+      <c r="B337" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="C337" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D337" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E337" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F337" s="5" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A338" s="2">
+        <v>337</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="C338" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D338" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E338" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F338" s="3" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A339" s="4">
+        <v>338</v>
+      </c>
+      <c r="B339" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="C339" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D339" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E339" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F339" s="5" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A340" s="2">
+        <v>339</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>739</v>
+      </c>
+      <c r="C340" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D340" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E340" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F340" s="3" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A341" s="4">
+        <v>340</v>
+      </c>
+      <c r="B341" s="5" t="s">
+        <v>741</v>
+      </c>
+      <c r="C341" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D341" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E341" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F341" s="5" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A342" s="2">
+        <v>341</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>743</v>
+      </c>
+      <c r="C342" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D342" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E342" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F342" s="3" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A343" s="4">
+        <v>342</v>
+      </c>
+      <c r="B343" s="5" t="s">
+        <v>745</v>
+      </c>
+      <c r="C343" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D343" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E343" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F343" s="5" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A344" s="2">
+        <v>343</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="C344" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="D344" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E344" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F344" s="3" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A345" s="4">
+        <v>344</v>
+      </c>
+      <c r="B345" s="5" t="s">
+        <v>750</v>
+      </c>
+      <c r="C345" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D345" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E345" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A346" s="2">
+        <v>345</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>752</v>
+      </c>
+      <c r="C346" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D346" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E346" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F346" s="3" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A347" s="4">
+        <v>346</v>
+      </c>
+      <c r="B347" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="C347" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D347" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E347" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F347" s="5" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A348" s="2">
+        <v>347</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="C348" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D348" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E348" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F348" s="3" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A349" s="4">
+        <v>348</v>
+      </c>
+      <c r="B349" s="5" t="s">
+        <v>758</v>
+      </c>
+      <c r="C349" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D349" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E349" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F349" s="5" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A350" s="2">
+        <v>349</v>
+      </c>
+      <c r="B350" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="C350" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D350" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E350" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F350" s="3" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A351" s="4">
+        <v>350</v>
+      </c>
+      <c r="B351" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="C351" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D351" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E351" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F351" s="5" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A352" s="2">
+        <v>351</v>
+      </c>
+      <c r="B352" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="C352" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D352" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E352" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F352" s="3" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A353" s="4">
+        <v>352</v>
+      </c>
+      <c r="B353" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="C353" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D353" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E353" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F353" s="5" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A354" s="2">
+        <v>353</v>
+      </c>
+      <c r="B354" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E354" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F354" s="3" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="355" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A355" s="4">
+        <v>354</v>
+      </c>
+      <c r="B355" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="C355" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="D355" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E355" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F355" s="5" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="356" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A356" s="2">
+        <v>355</v>
+      </c>
+      <c r="B356" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E356" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F356" s="3" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A357" s="4">
+        <v>356</v>
+      </c>
+      <c r="B357" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="C357" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="D357" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E357" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F357" s="5" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A358" s="2">
+        <v>357</v>
+      </c>
+      <c r="B358" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E358" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F358" s="3" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A359" s="4">
+        <v>358</v>
+      </c>
+      <c r="B359" s="5" t="s">
+        <v>779</v>
+      </c>
+      <c r="C359" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D359" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E359" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F359" s="5" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A360" s="2">
+        <v>359</v>
+      </c>
+      <c r="B360" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E360" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F360" s="3" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A361" s="4">
+        <v>360</v>
+      </c>
+      <c r="B361" s="5" t="s">
+        <v>784</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D361" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E361" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F361" s="5" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A362" s="2">
+        <v>361</v>
+      </c>
+      <c r="B362" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C362" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E362" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F362" s="3" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A363" s="4">
+        <v>362</v>
+      </c>
+      <c r="B363" s="5" t="s">
+        <v>788</v>
+      </c>
+      <c r="C363" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D363" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E363" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F363" s="5" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="364" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A364" s="2">
+        <v>363</v>
+      </c>
+      <c r="B364" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F364" s="3" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="365" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A365" s="4">
+        <v>364</v>
+      </c>
+      <c r="B365" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="C365" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="D365" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E365" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F365" s="5" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="366" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A366" s="2">
+        <v>365</v>
+      </c>
+      <c r="B366" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="C366" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E366" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F366" s="3" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="367" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A367" s="4">
+        <v>366</v>
+      </c>
+      <c r="B367" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="C367" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D367" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E367" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F367" s="5" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="368" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A368" s="2">
+        <v>367</v>
+      </c>
+      <c r="B368" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="C368" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D368" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E368" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F368" s="3" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A369" s="4">
+        <v>368</v>
+      </c>
+      <c r="B369" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D369" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E369" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F369" s="5" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A370" s="2">
+        <v>369</v>
+      </c>
+      <c r="B370" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="C370" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D370" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E370" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F370" s="3" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A371" s="4">
+        <v>370</v>
+      </c>
+      <c r="B371" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="C371" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D371" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E371" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F371" s="5" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A372" s="2">
+        <v>371</v>
+      </c>
+      <c r="B372" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="C372" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D372" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E372" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F372" s="3" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A373" s="4">
+        <v>372</v>
+      </c>
+      <c r="B373" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="C373" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D373" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E373" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F373" s="5" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A374" s="2">
+        <v>373</v>
+      </c>
+      <c r="B374" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="C374" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D374" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E374" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F374" s="3" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A375" s="4">
+        <v>374</v>
+      </c>
+      <c r="B375" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="C375" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D375" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E375" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F375" s="5" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A376" s="2">
+        <v>375</v>
+      </c>
+      <c r="B376" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="C376" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D376" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E376" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F376" s="3" t="s">
+        <v>816</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Revert "Add MTA descriptions and post-bind Risk ID assertions across tests"
This reverts commit 007184fdfc2d0cc0d320e17f58a172eb0589686a.
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="523">
   <si>
     <t>Run #</t>
   </si>
@@ -1580,888 +1580,6 @@
   </si>
   <si>
     <t>13/05/2026, 15:27:19</t>
-  </si>
-  <si>
-    <t>DA-MLI-537284133</t>
-  </si>
-  <si>
-    <t>13/05/2026, 15:54:39</t>
-  </si>
-  <si>
-    <t>DA-MLI-537285133</t>
-  </si>
-  <si>
-    <t>13/05/2026, 15:56:51</t>
-  </si>
-  <si>
-    <t>DA-MLI-080082134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 11:49:36</t>
-  </si>
-  <si>
-    <t>CP-MLI-062655134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 13:23:14</t>
-  </si>
-  <si>
-    <t>DA-MLI-080091134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 13:48:32</t>
-  </si>
-  <si>
-    <t>DA-MLI-080095134</t>
-  </si>
-  <si>
-    <t>TC_REG_042 | Cancel and reissue date today then MTA effective date cannot be yesterday</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:02:01</t>
-  </si>
-  <si>
-    <t>DA-MLI-080099134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:07:56</t>
-  </si>
-  <si>
-    <t>DA-MLI-080102134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:14:00</t>
-  </si>
-  <si>
-    <t>DA-MLI-080105134</t>
-  </si>
-  <si>
-    <t>TC_REG_043 | Create MTA then Cancel and Reissue then Create MTA</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:28:08</t>
-  </si>
-  <si>
-    <t>DA-MLI-080112134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:40:30</t>
-  </si>
-  <si>
-    <t>DA-MLI-537294134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:52:15</t>
-  </si>
-  <si>
-    <t>DA-MLI-537296134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 14:55:48</t>
-  </si>
-  <si>
-    <t>CP-MLI-062657134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:17:43</t>
-  </si>
-  <si>
-    <t>CP-MLI-062659134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:19:11</t>
-  </si>
-  <si>
-    <t>DA-MLI-062679134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:24:32</t>
-  </si>
-  <si>
-    <t>DA-MLI-062688134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:27:00</t>
-  </si>
-  <si>
-    <t>DA-MLI-062705134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:30:33</t>
-  </si>
-  <si>
-    <t>DA-MLI-080120134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 15:43:05</t>
-  </si>
-  <si>
-    <t>CP-NI-080127134</t>
-  </si>
-  <si>
-    <t>DT-MLIS-DF25.5.0 | CR-237340 |TC_34_S6_Verify Cancellation premiums are applied to the appropriate intermediary when user change the Intermediary Legal Entity on MTA _NB&gt;CRN&gt;MTA_Cancel the Policy Mid-term_NI commercial_Broker portal</t>
-  </si>
-  <si>
-    <t>14/05/2026, 17:19:06</t>
-  </si>
-  <si>
-    <t>CP-NI-080129134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 17:23:09</t>
-  </si>
-  <si>
-    <t>CP-NI-080132134</t>
-  </si>
-  <si>
-    <t>14/05/2026, 17:28:52</t>
-  </si>
-  <si>
-    <t>CP-NI-080495138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:32:40</t>
-  </si>
-  <si>
-    <t>CP-NI-080497138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:37:13</t>
-  </si>
-  <si>
-    <t>CP-NI-080499138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:41:41</t>
-  </si>
-  <si>
-    <t>CP-NI-080501138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:45:06</t>
-  </si>
-  <si>
-    <t>CP-NI-080503138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:49:18</t>
-  </si>
-  <si>
-    <t>CP-NI-080506138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 08:53:09</t>
-  </si>
-  <si>
-    <t>CP-NI-080510138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:02:42</t>
-  </si>
-  <si>
-    <t>CP-NI-080513138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:08:11</t>
-  </si>
-  <si>
-    <t>CP-NI-080516138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:12:55</t>
-  </si>
-  <si>
-    <t>CP-NI-080517138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:14:47</t>
-  </si>
-  <si>
-    <t>CP-NI-080520138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:21:54</t>
-  </si>
-  <si>
-    <t>CP-NI-080523138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:26:08</t>
-  </si>
-  <si>
-    <t>CP-NI-080526138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:31:55</t>
-  </si>
-  <si>
-    <t>CP-NI-080528138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:37:44</t>
-  </si>
-  <si>
-    <t>CP-NI-080532138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:46:06</t>
-  </si>
-  <si>
-    <t>CP-NI-080535138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 09:53:45</t>
-  </si>
-  <si>
-    <t>CP-NI-080538138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:02:54</t>
-  </si>
-  <si>
-    <t>CP-NI-080541138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:09:12</t>
-  </si>
-  <si>
-    <t>CP-NI-080544138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:15:18</t>
-  </si>
-  <si>
-    <t>CP-NI-080547138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:20:19</t>
-  </si>
-  <si>
-    <t>CP-NI-080550138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:27:05</t>
-  </si>
-  <si>
-    <t>CP-NI-080553138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:32:16</t>
-  </si>
-  <si>
-    <t>CP-NI-080555138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:35:09</t>
-  </si>
-  <si>
-    <t>CP-NI-080558138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:41:30</t>
-  </si>
-  <si>
-    <t>CP-NI-080561138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 10:51:51</t>
-  </si>
-  <si>
-    <t>CP-NI-080564138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:00:13</t>
-  </si>
-  <si>
-    <t>CP-NI-062979138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:04:14</t>
-  </si>
-  <si>
-    <t>CP-NI-080567138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:17:49</t>
-  </si>
-  <si>
-    <t>CP-NI-080570138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:22:21</t>
-  </si>
-  <si>
-    <t>CP-NI-080572138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:24:42</t>
-  </si>
-  <si>
-    <t>CP-NI-080575138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:29:27</t>
-  </si>
-  <si>
-    <t>CP-NI-080577138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:32:10</t>
-  </si>
-  <si>
-    <t>CP-NI-080580138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:38:36</t>
-  </si>
-  <si>
-    <t>CP-NI-080583138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:43:49</t>
-  </si>
-  <si>
-    <t>CP-NI-080586138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:48:56</t>
-  </si>
-  <si>
-    <t>CP-NI-080589138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 11:55:02</t>
-  </si>
-  <si>
-    <t>CP-NI-080593138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:02:30</t>
-  </si>
-  <si>
-    <t>CP-NI-080596138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:08:40</t>
-  </si>
-  <si>
-    <t>CP-NI-080599138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:14:51</t>
-  </si>
-  <si>
-    <t>CP-NI-080602138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:21:46</t>
-  </si>
-  <si>
-    <t>CP-NI-080605138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:27:44</t>
-  </si>
-  <si>
-    <t>CP-NI-080606138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:29:49</t>
-  </si>
-  <si>
-    <t>CP-NI-080608138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 12:33:04</t>
-  </si>
-  <si>
-    <t>DA-MLI-080624138</t>
-  </si>
-  <si>
-    <t>TC_REG_045 | Source Submission -&gt; Change of Limit of Indemnity updates Limit of Indemnity after refresh</t>
-  </si>
-  <si>
-    <t>18/05/2026, 13:45:16</t>
-  </si>
-  <si>
-    <t>DA-MLI-080626138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 13:51:05</t>
-  </si>
-  <si>
-    <t>DA-MLI-080628138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:00:59</t>
-  </si>
-  <si>
-    <t>DA-MLI-080672138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:11:05</t>
-  </si>
-  <si>
-    <t>DA-MLI-080717138</t>
-  </si>
-  <si>
-    <t>TC_REG_045 | Clear MTA flow on a live policy</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:25:34</t>
-  </si>
-  <si>
-    <t>DA-MLI-080719138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:27:14</t>
-  </si>
-  <si>
-    <t>DA-MLI-080722138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:29:04</t>
-  </si>
-  <si>
-    <t>DA-MLI-080726138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:33:21</t>
-  </si>
-  <si>
-    <t>DA-MLI-080728138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:35:33</t>
-  </si>
-  <si>
-    <t>DA-MLI-080729138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:38:35</t>
-  </si>
-  <si>
-    <t>DA-MLI-080732138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:43:25</t>
-  </si>
-  <si>
-    <t>DA-MLI-080735138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:46:28</t>
-  </si>
-  <si>
-    <t>DA-MLI-080737138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:51:05</t>
-  </si>
-  <si>
-    <t>DA-MLI-080738138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:52:59</t>
-  </si>
-  <si>
-    <t>DA-MLI-080741138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:55:59</t>
-  </si>
-  <si>
-    <t>DA-MLI-080743138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 14:59:36</t>
-  </si>
-  <si>
-    <t>DA-MLI-080744138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:02:46</t>
-  </si>
-  <si>
-    <t>DA-MLI-080745138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:04:44</t>
-  </si>
-  <si>
-    <t>DA-MLI-080747138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:09:36</t>
-  </si>
-  <si>
-    <t>DA-MLI-080750138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:14:18</t>
-  </si>
-  <si>
-    <t>DA-MLI-080753138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:20:32</t>
-  </si>
-  <si>
-    <t>DA-MLI-080755138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:23:53</t>
-  </si>
-  <si>
-    <t>DA-MLI-080759138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 15:29:58</t>
-  </si>
-  <si>
-    <t>DA-MLI-080769138</t>
-  </si>
-  <si>
-    <t>TC_REG_046 | Create MTA without bind, assert Insurance Policies (0) and Quotes (1), open Quote</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:17:48</t>
-  </si>
-  <si>
-    <t>DA-MLI-080770138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:21:29</t>
-  </si>
-  <si>
-    <t>DA-MLI-080773138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:25:30</t>
-  </si>
-  <si>
-    <t>CP-NI-080776138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:35:28</t>
-  </si>
-  <si>
-    <t>CP-NI-080780138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:42:16</t>
-  </si>
-  <si>
-    <t>CP-NI-080783138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:48:31</t>
-  </si>
-  <si>
-    <t>CP-NI-080787138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:54:49</t>
-  </si>
-  <si>
-    <t>CP-NI-080789138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 16:57:11</t>
-  </si>
-  <si>
-    <t>CP-NI-080794138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 17:09:08</t>
-  </si>
-  <si>
-    <t>CP-NI-080798138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 17:15:09</t>
-  </si>
-  <si>
-    <t>CP-NI-063006138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 17:59:05</t>
-  </si>
-  <si>
-    <t>CP-NI-063005138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 18:00:36</t>
-  </si>
-  <si>
-    <t>CP-NI-080817138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 18:02:27</t>
-  </si>
-  <si>
-    <t>CP-NI-080823138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 18:07:26</t>
-  </si>
-  <si>
-    <t>CP-NI-080828138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 18:15:44</t>
-  </si>
-  <si>
-    <t>CP-NI-080835138</t>
-  </si>
-  <si>
-    <t>18/05/2026, 18:26:54</t>
-  </si>
-  <si>
-    <t>CP-NI-080956139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:10:46</t>
-  </si>
-  <si>
-    <t>CP-NI-080961139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:19:59</t>
-  </si>
-  <si>
-    <t>CP-NI-080969139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:32:28</t>
-  </si>
-  <si>
-    <t>CP-NI-080971139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:35:48</t>
-  </si>
-  <si>
-    <t>CP-NI-080973139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:38:51</t>
-  </si>
-  <si>
-    <t>CP-NI-080974139</t>
-  </si>
-  <si>
-    <t>19/05/2026, 15:40:50</t>
-  </si>
-  <si>
-    <t>DA-MLI-063700140</t>
-  </si>
-  <si>
-    <t>TC_BDX_005_NB_MTA | Create NB-MTA (Mid-Term Adjustment) on a live policy</t>
-  </si>
-  <si>
-    <t>20/05/2026, 10:04:01</t>
-  </si>
-  <si>
-    <t>DA-MLI-081093140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 10:06:43</t>
-  </si>
-  <si>
-    <t>DA-MLI-081094140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 10:10:22</t>
-  </si>
-  <si>
-    <t>DA-MLI-081095140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 10:10:24</t>
-  </si>
-  <si>
-    <t>DA-MLI-081098140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 10:13:48</t>
-  </si>
-  <si>
-    <t>CP-MLI-081106140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:44:59</t>
-  </si>
-  <si>
-    <t>DA-MLI-063836140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:50:06</t>
-  </si>
-  <si>
-    <t>DA-MLI-063843140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:55:02</t>
-  </si>
-  <si>
-    <t>DA-MLI-063847140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:57:13</t>
-  </si>
-  <si>
-    <t>CP-MLI-063851140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:59:02</t>
-  </si>
-  <si>
-    <t>DA-MLI-063852140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 12:59:50</t>
-  </si>
-  <si>
-    <t>DA-MLI-081125140</t>
-  </si>
-  <si>
-    <t>TC_REG_047 | Save at quotes, verify SF related counts, resume and issue policy</t>
-  </si>
-  <si>
-    <t>20/05/2026, 13:37:39</t>
-  </si>
-  <si>
-    <t>DA-MLI-081127140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 13:46:16</t>
-  </si>
-  <si>
-    <t>DA-MLI-081129140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 13:55:05</t>
-  </si>
-  <si>
-    <t>DA-MLI-081130140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 14:01:19</t>
-  </si>
-  <si>
-    <t>DA-MLI-081133140</t>
-  </si>
-  <si>
-    <t>TC_REG_048 | NB-MTA validate Edit Terms Discount + Update Premium fallback and complete bind</t>
-  </si>
-  <si>
-    <t>20/05/2026, 14:43:34</t>
-  </si>
-  <si>
-    <t>DA-MLI-081134140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 14:50:38</t>
-  </si>
-  <si>
-    <t>DA-MLI-081136140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 14:54:34</t>
-  </si>
-  <si>
-    <t>DA-MLI-081138140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 15:00:32</t>
-  </si>
-  <si>
-    <t>DA-MLI-081141140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 15:11:13</t>
-  </si>
-  <si>
-    <t>DA-MLI-081143140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 15:21:12</t>
-  </si>
-  <si>
-    <t>DA-MLI-081148140</t>
-  </si>
-  <si>
-    <t>TC_REG_049 | Create NB then update discount on Quotes tab and continue quote in Salesforce</t>
-  </si>
-  <si>
-    <t>20/05/2026, 15:46:33</t>
-  </si>
-  <si>
-    <t>DA-MLI-063952140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 17:50:06</t>
-  </si>
-  <si>
-    <t>DA-MLI-063954140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 17:53:05</t>
-  </si>
-  <si>
-    <t>DA-MLI-063955140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 17:54:55</t>
-  </si>
-  <si>
-    <t>DA-MLI-063956140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 17:59:42</t>
-  </si>
-  <si>
-    <t>DA-MLI-063967140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 18:40:06</t>
-  </si>
-  <si>
-    <t>DA-MLI-063971140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 18:53:13</t>
-  </si>
-  <si>
-    <t>DA-MLI-063974140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 18:59:59</t>
-  </si>
-  <si>
-    <t>DA-MLI-063977140</t>
-  </si>
-  <si>
-    <t>20/05/2026, 19:09:16</t>
-  </si>
-  <si>
-    <t>DA-MLI-081322141</t>
-  </si>
-  <si>
-    <t>21/05/2026, 15:55:11</t>
-  </si>
-  <si>
-    <t>DA-MLI-081332141</t>
-  </si>
-  <si>
-    <t>21/05/2026, 16:00:50</t>
-  </si>
-  <si>
-    <t>DA-MLI-081334141</t>
-  </si>
-  <si>
-    <t>21/05/2026, 16:02:27</t>
   </si>
 </sst>
 </file>
@@ -2895,7 +2013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F376"/>
+  <dimension ref="A1:F234"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -7586,2846 +6704,6 @@
         <v>522</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A235" s="4">
-        <v>234</v>
-      </c>
-      <c r="B235" s="5" t="s">
-        <v>523</v>
-      </c>
-      <c r="C235" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D235" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E235" s="5" t="s">
-        <v>491</v>
-      </c>
-      <c r="F235" s="5" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A236" s="2">
-        <v>235</v>
-      </c>
-      <c r="B236" s="3" t="s">
-        <v>525</v>
-      </c>
-      <c r="C236" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D236" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E236" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="F236" s="3" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A237" s="4">
-        <v>236</v>
-      </c>
-      <c r="B237" s="5" t="s">
-        <v>527</v>
-      </c>
-      <c r="C237" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D237" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E237" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F237" s="5" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A238" s="2">
-        <v>237</v>
-      </c>
-      <c r="B238" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="C238" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D238" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E238" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F238" s="3" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A239" s="4">
-        <v>238</v>
-      </c>
-      <c r="B239" s="5" t="s">
-        <v>531</v>
-      </c>
-      <c r="C239" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D239" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E239" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F239" s="5" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A240" s="2">
-        <v>239</v>
-      </c>
-      <c r="B240" s="3" t="s">
-        <v>533</v>
-      </c>
-      <c r="C240" s="3" t="s">
-        <v>534</v>
-      </c>
-      <c r="D240" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E240" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F240" s="3" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A241" s="4">
-        <v>240</v>
-      </c>
-      <c r="B241" s="5" t="s">
-        <v>536</v>
-      </c>
-      <c r="C241" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="D241" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E241" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F241" s="5" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A242" s="2">
-        <v>241</v>
-      </c>
-      <c r="B242" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="C242" s="3" t="s">
-        <v>534</v>
-      </c>
-      <c r="D242" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E242" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F242" s="3" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A243" s="4">
-        <v>242</v>
-      </c>
-      <c r="B243" s="5" t="s">
-        <v>540</v>
-      </c>
-      <c r="C243" s="5" t="s">
-        <v>541</v>
-      </c>
-      <c r="D243" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E243" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F243" s="5" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A244" s="2">
-        <v>243</v>
-      </c>
-      <c r="B244" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="C244" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="D244" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E244" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F244" s="3" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A245" s="4">
-        <v>244</v>
-      </c>
-      <c r="B245" s="5" t="s">
-        <v>545</v>
-      </c>
-      <c r="C245" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D245" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E245" s="5" t="s">
-        <v>491</v>
-      </c>
-      <c r="F245" s="5" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A246" s="2">
-        <v>245</v>
-      </c>
-      <c r="B246" s="3" t="s">
-        <v>547</v>
-      </c>
-      <c r="C246" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D246" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E246" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="F246" s="3" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A247" s="4">
-        <v>246</v>
-      </c>
-      <c r="B247" s="5" t="s">
-        <v>549</v>
-      </c>
-      <c r="C247" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D247" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E247" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F247" s="5" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A248" s="2">
-        <v>247</v>
-      </c>
-      <c r="B248" s="3" t="s">
-        <v>551</v>
-      </c>
-      <c r="C248" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D248" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E248" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F248" s="3" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A249" s="4">
-        <v>248</v>
-      </c>
-      <c r="B249" s="5" t="s">
-        <v>553</v>
-      </c>
-      <c r="C249" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D249" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E249" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F249" s="5" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A250" s="2">
-        <v>249</v>
-      </c>
-      <c r="B250" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="C250" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D250" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E250" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F250" s="3" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A251" s="4">
-        <v>250</v>
-      </c>
-      <c r="B251" s="5" t="s">
-        <v>557</v>
-      </c>
-      <c r="C251" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D251" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E251" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F251" s="5" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A252" s="2">
-        <v>251</v>
-      </c>
-      <c r="B252" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="C252" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D252" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E252" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F252" s="3" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A253" s="4">
-        <v>252</v>
-      </c>
-      <c r="B253" s="5" t="s">
-        <v>561</v>
-      </c>
-      <c r="C253" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D253" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E253" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F253" s="5" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A254" s="2">
-        <v>253</v>
-      </c>
-      <c r="B254" s="3" t="s">
-        <v>564</v>
-      </c>
-      <c r="C254" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D254" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E254" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F254" s="3" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A255" s="4">
-        <v>254</v>
-      </c>
-      <c r="B255" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="C255" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D255" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E255" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F255" s="5" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A256" s="2">
-        <v>255</v>
-      </c>
-      <c r="B256" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="C256" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D256" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E256" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F256" s="3" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A257" s="4">
-        <v>256</v>
-      </c>
-      <c r="B257" s="5" t="s">
-        <v>570</v>
-      </c>
-      <c r="C257" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D257" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E257" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F257" s="5" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A258" s="2">
-        <v>257</v>
-      </c>
-      <c r="B258" s="3" t="s">
-        <v>572</v>
-      </c>
-      <c r="C258" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D258" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E258" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F258" s="3" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A259" s="4">
-        <v>258</v>
-      </c>
-      <c r="B259" s="5" t="s">
-        <v>574</v>
-      </c>
-      <c r="C259" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D259" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E259" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F259" s="5" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A260" s="2">
-        <v>259</v>
-      </c>
-      <c r="B260" s="3" t="s">
-        <v>576</v>
-      </c>
-      <c r="C260" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D260" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E260" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F260" s="3" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A261" s="4">
-        <v>260</v>
-      </c>
-      <c r="B261" s="5" t="s">
-        <v>578</v>
-      </c>
-      <c r="C261" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D261" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E261" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F261" s="5" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A262" s="2">
-        <v>261</v>
-      </c>
-      <c r="B262" s="3" t="s">
-        <v>580</v>
-      </c>
-      <c r="C262" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D262" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E262" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F262" s="3" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A263" s="4">
-        <v>262</v>
-      </c>
-      <c r="B263" s="5" t="s">
-        <v>582</v>
-      </c>
-      <c r="C263" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D263" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E263" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F263" s="5" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A264" s="2">
-        <v>263</v>
-      </c>
-      <c r="B264" s="3" t="s">
-        <v>584</v>
-      </c>
-      <c r="C264" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D264" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E264" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F264" s="3" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A265" s="4">
-        <v>264</v>
-      </c>
-      <c r="B265" s="5" t="s">
-        <v>586</v>
-      </c>
-      <c r="C265" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D265" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E265" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F265" s="5" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A266" s="2">
-        <v>265</v>
-      </c>
-      <c r="B266" s="3" t="s">
-        <v>588</v>
-      </c>
-      <c r="C266" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D266" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E266" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F266" s="3" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A267" s="4">
-        <v>266</v>
-      </c>
-      <c r="B267" s="5" t="s">
-        <v>590</v>
-      </c>
-      <c r="C267" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D267" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E267" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F267" s="5" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A268" s="2">
-        <v>267</v>
-      </c>
-      <c r="B268" s="3" t="s">
-        <v>592</v>
-      </c>
-      <c r="C268" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D268" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E268" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F268" s="3" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A269" s="4">
-        <v>268</v>
-      </c>
-      <c r="B269" s="5" t="s">
-        <v>594</v>
-      </c>
-      <c r="C269" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D269" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E269" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F269" s="5" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A270" s="2">
-        <v>269</v>
-      </c>
-      <c r="B270" s="3" t="s">
-        <v>596</v>
-      </c>
-      <c r="C270" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D270" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E270" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F270" s="3" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A271" s="4">
-        <v>270</v>
-      </c>
-      <c r="B271" s="5" t="s">
-        <v>598</v>
-      </c>
-      <c r="C271" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D271" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E271" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F271" s="5" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A272" s="2">
-        <v>271</v>
-      </c>
-      <c r="B272" s="3" t="s">
-        <v>600</v>
-      </c>
-      <c r="C272" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D272" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E272" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F272" s="3" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A273" s="4">
-        <v>272</v>
-      </c>
-      <c r="B273" s="5" t="s">
-        <v>602</v>
-      </c>
-      <c r="C273" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D273" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E273" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F273" s="5" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A274" s="2">
-        <v>273</v>
-      </c>
-      <c r="B274" s="3" t="s">
-        <v>604</v>
-      </c>
-      <c r="C274" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D274" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E274" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F274" s="3" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A275" s="4">
-        <v>274</v>
-      </c>
-      <c r="B275" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="C275" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D275" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E275" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F275" s="5" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A276" s="2">
-        <v>275</v>
-      </c>
-      <c r="B276" s="3" t="s">
-        <v>608</v>
-      </c>
-      <c r="C276" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D276" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E276" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F276" s="3" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A277" s="4">
-        <v>276</v>
-      </c>
-      <c r="B277" s="5" t="s">
-        <v>610</v>
-      </c>
-      <c r="C277" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D277" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E277" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F277" s="5" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A278" s="2">
-        <v>277</v>
-      </c>
-      <c r="B278" s="3" t="s">
-        <v>612</v>
-      </c>
-      <c r="C278" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D278" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E278" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F278" s="3" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A279" s="4">
-        <v>278</v>
-      </c>
-      <c r="B279" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="C279" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D279" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E279" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F279" s="5" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A280" s="2">
-        <v>279</v>
-      </c>
-      <c r="B280" s="3" t="s">
-        <v>616</v>
-      </c>
-      <c r="C280" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D280" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E280" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F280" s="3" t="s">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A281" s="4">
-        <v>280</v>
-      </c>
-      <c r="B281" s="5" t="s">
-        <v>618</v>
-      </c>
-      <c r="C281" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D281" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E281" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F281" s="5" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A282" s="2">
-        <v>281</v>
-      </c>
-      <c r="B282" s="3" t="s">
-        <v>620</v>
-      </c>
-      <c r="C282" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D282" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E282" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F282" s="3" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A283" s="4">
-        <v>282</v>
-      </c>
-      <c r="B283" s="5" t="s">
-        <v>622</v>
-      </c>
-      <c r="C283" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D283" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E283" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F283" s="5" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A284" s="2">
-        <v>283</v>
-      </c>
-      <c r="B284" s="3" t="s">
-        <v>624</v>
-      </c>
-      <c r="C284" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D284" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E284" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F284" s="3" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A285" s="4">
-        <v>284</v>
-      </c>
-      <c r="B285" s="5" t="s">
-        <v>626</v>
-      </c>
-      <c r="C285" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D285" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E285" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F285" s="5" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A286" s="2">
-        <v>285</v>
-      </c>
-      <c r="B286" s="3" t="s">
-        <v>628</v>
-      </c>
-      <c r="C286" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D286" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E286" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F286" s="3" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A287" s="4">
-        <v>286</v>
-      </c>
-      <c r="B287" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="C287" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D287" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E287" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F287" s="5" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A288" s="2">
-        <v>287</v>
-      </c>
-      <c r="B288" s="3" t="s">
-        <v>632</v>
-      </c>
-      <c r="C288" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D288" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E288" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F288" s="3" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A289" s="4">
-        <v>288</v>
-      </c>
-      <c r="B289" s="5" t="s">
-        <v>634</v>
-      </c>
-      <c r="C289" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D289" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E289" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F289" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A290" s="2">
-        <v>289</v>
-      </c>
-      <c r="B290" s="3" t="s">
-        <v>636</v>
-      </c>
-      <c r="C290" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D290" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E290" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F290" s="3" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A291" s="4">
-        <v>290</v>
-      </c>
-      <c r="B291" s="5" t="s">
-        <v>638</v>
-      </c>
-      <c r="C291" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D291" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E291" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F291" s="5" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A292" s="2">
-        <v>291</v>
-      </c>
-      <c r="B292" s="3" t="s">
-        <v>640</v>
-      </c>
-      <c r="C292" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D292" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E292" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F292" s="3" t="s">
-        <v>641</v>
-      </c>
-    </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A293" s="4">
-        <v>292</v>
-      </c>
-      <c r="B293" s="5" t="s">
-        <v>642</v>
-      </c>
-      <c r="C293" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D293" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E293" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F293" s="5" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A294" s="2">
-        <v>293</v>
-      </c>
-      <c r="B294" s="3" t="s">
-        <v>644</v>
-      </c>
-      <c r="C294" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D294" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E294" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F294" s="3" t="s">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A295" s="4">
-        <v>294</v>
-      </c>
-      <c r="B295" s="5" t="s">
-        <v>646</v>
-      </c>
-      <c r="C295" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D295" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E295" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F295" s="5" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A296" s="2">
-        <v>295</v>
-      </c>
-      <c r="B296" s="3" t="s">
-        <v>648</v>
-      </c>
-      <c r="C296" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D296" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E296" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F296" s="3" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A297" s="4">
-        <v>296</v>
-      </c>
-      <c r="B297" s="5" t="s">
-        <v>650</v>
-      </c>
-      <c r="C297" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D297" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E297" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F297" s="5" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A298" s="2">
-        <v>297</v>
-      </c>
-      <c r="B298" s="3" t="s">
-        <v>652</v>
-      </c>
-      <c r="C298" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D298" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E298" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F298" s="3" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A299" s="4">
-        <v>298</v>
-      </c>
-      <c r="B299" s="5" t="s">
-        <v>654</v>
-      </c>
-      <c r="C299" s="5" t="s">
-        <v>655</v>
-      </c>
-      <c r="D299" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E299" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F299" s="5" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A300" s="2">
-        <v>299</v>
-      </c>
-      <c r="B300" s="3" t="s">
-        <v>657</v>
-      </c>
-      <c r="C300" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="D300" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E300" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F300" s="3" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A301" s="4">
-        <v>300</v>
-      </c>
-      <c r="B301" s="5" t="s">
-        <v>659</v>
-      </c>
-      <c r="C301" s="5" t="s">
-        <v>655</v>
-      </c>
-      <c r="D301" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E301" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F301" s="5" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A302" s="2">
-        <v>301</v>
-      </c>
-      <c r="B302" s="3" t="s">
-        <v>661</v>
-      </c>
-      <c r="C302" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="D302" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E302" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F302" s="3" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A303" s="4">
-        <v>302</v>
-      </c>
-      <c r="B303" s="5" t="s">
-        <v>663</v>
-      </c>
-      <c r="C303" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D303" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E303" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F303" s="5" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A304" s="2">
-        <v>303</v>
-      </c>
-      <c r="B304" s="3" t="s">
-        <v>666</v>
-      </c>
-      <c r="C304" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D304" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E304" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F304" s="3" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A305" s="4">
-        <v>304</v>
-      </c>
-      <c r="B305" s="5" t="s">
-        <v>668</v>
-      </c>
-      <c r="C305" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D305" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E305" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F305" s="5" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A306" s="2">
-        <v>305</v>
-      </c>
-      <c r="B306" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="C306" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D306" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E306" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F306" s="3" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A307" s="4">
-        <v>306</v>
-      </c>
-      <c r="B307" s="5" t="s">
-        <v>672</v>
-      </c>
-      <c r="C307" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D307" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E307" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F307" s="5" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A308" s="2">
-        <v>307</v>
-      </c>
-      <c r="B308" s="3" t="s">
-        <v>674</v>
-      </c>
-      <c r="C308" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D308" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E308" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F308" s="3" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A309" s="4">
-        <v>308</v>
-      </c>
-      <c r="B309" s="5" t="s">
-        <v>676</v>
-      </c>
-      <c r="C309" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D309" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E309" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F309" s="5" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A310" s="2">
-        <v>309</v>
-      </c>
-      <c r="B310" s="3" t="s">
-        <v>678</v>
-      </c>
-      <c r="C310" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D310" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E310" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F310" s="3" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A311" s="4">
-        <v>310</v>
-      </c>
-      <c r="B311" s="5" t="s">
-        <v>680</v>
-      </c>
-      <c r="C311" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D311" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E311" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F311" s="5" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A312" s="2">
-        <v>311</v>
-      </c>
-      <c r="B312" s="3" t="s">
-        <v>682</v>
-      </c>
-      <c r="C312" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D312" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E312" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F312" s="3" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A313" s="4">
-        <v>312</v>
-      </c>
-      <c r="B313" s="5" t="s">
-        <v>684</v>
-      </c>
-      <c r="C313" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D313" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E313" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F313" s="5" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A314" s="2">
-        <v>313</v>
-      </c>
-      <c r="B314" s="3" t="s">
-        <v>686</v>
-      </c>
-      <c r="C314" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D314" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E314" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F314" s="3" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A315" s="4">
-        <v>314</v>
-      </c>
-      <c r="B315" s="5" t="s">
-        <v>688</v>
-      </c>
-      <c r="C315" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D315" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E315" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F315" s="5" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A316" s="2">
-        <v>315</v>
-      </c>
-      <c r="B316" s="3" t="s">
-        <v>690</v>
-      </c>
-      <c r="C316" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D316" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E316" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F316" s="3" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A317" s="4">
-        <v>316</v>
-      </c>
-      <c r="B317" s="5" t="s">
-        <v>692</v>
-      </c>
-      <c r="C317" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D317" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E317" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F317" s="5" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A318" s="2">
-        <v>317</v>
-      </c>
-      <c r="B318" s="3" t="s">
-        <v>694</v>
-      </c>
-      <c r="C318" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D318" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E318" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F318" s="3" t="s">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A319" s="4">
-        <v>318</v>
-      </c>
-      <c r="B319" s="5" t="s">
-        <v>696</v>
-      </c>
-      <c r="C319" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D319" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E319" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F319" s="5" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A320" s="2">
-        <v>319</v>
-      </c>
-      <c r="B320" s="3" t="s">
-        <v>698</v>
-      </c>
-      <c r="C320" s="3" t="s">
-        <v>664</v>
-      </c>
-      <c r="D320" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E320" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F320" s="3" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A321" s="4">
-        <v>320</v>
-      </c>
-      <c r="B321" s="5" t="s">
-        <v>700</v>
-      </c>
-      <c r="C321" s="5" t="s">
-        <v>664</v>
-      </c>
-      <c r="D321" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E321" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F321" s="5" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A322" s="2">
-        <v>321</v>
-      </c>
-      <c r="B322" s="3" t="s">
-        <v>702</v>
-      </c>
-      <c r="C322" s="3" t="s">
-        <v>703</v>
-      </c>
-      <c r="D322" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E322" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F322" s="3" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A323" s="4">
-        <v>322</v>
-      </c>
-      <c r="B323" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="C323" s="5" t="s">
-        <v>703</v>
-      </c>
-      <c r="D323" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E323" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F323" s="5" t="s">
-        <v>706</v>
-      </c>
-    </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A324" s="2">
-        <v>323</v>
-      </c>
-      <c r="B324" s="3" t="s">
-        <v>707</v>
-      </c>
-      <c r="C324" s="3" t="s">
-        <v>703</v>
-      </c>
-      <c r="D324" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E324" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F324" s="3" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A325" s="4">
-        <v>324</v>
-      </c>
-      <c r="B325" s="5" t="s">
-        <v>709</v>
-      </c>
-      <c r="C325" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D325" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E325" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F325" s="5" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A326" s="2">
-        <v>325</v>
-      </c>
-      <c r="B326" s="3" t="s">
-        <v>711</v>
-      </c>
-      <c r="C326" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D326" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E326" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F326" s="3" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A327" s="4">
-        <v>326</v>
-      </c>
-      <c r="B327" s="5" t="s">
-        <v>713</v>
-      </c>
-      <c r="C327" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D327" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E327" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F327" s="5" t="s">
-        <v>714</v>
-      </c>
-    </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A328" s="2">
-        <v>327</v>
-      </c>
-      <c r="B328" s="3" t="s">
-        <v>715</v>
-      </c>
-      <c r="C328" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D328" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E328" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F328" s="3" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A329" s="4">
-        <v>328</v>
-      </c>
-      <c r="B329" s="5" t="s">
-        <v>717</v>
-      </c>
-      <c r="C329" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D329" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E329" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F329" s="5" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A330" s="2">
-        <v>329</v>
-      </c>
-      <c r="B330" s="3" t="s">
-        <v>719</v>
-      </c>
-      <c r="C330" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D330" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E330" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F330" s="3" t="s">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A331" s="4">
-        <v>330</v>
-      </c>
-      <c r="B331" s="5" t="s">
-        <v>721</v>
-      </c>
-      <c r="C331" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D331" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E331" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F331" s="5" t="s">
-        <v>722</v>
-      </c>
-    </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A332" s="2">
-        <v>331</v>
-      </c>
-      <c r="B332" s="3" t="s">
-        <v>723</v>
-      </c>
-      <c r="C332" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D332" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E332" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F332" s="3" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A333" s="4">
-        <v>332</v>
-      </c>
-      <c r="B333" s="5" t="s">
-        <v>725</v>
-      </c>
-      <c r="C333" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D333" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E333" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F333" s="5" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A334" s="2">
-        <v>333</v>
-      </c>
-      <c r="B334" s="3" t="s">
-        <v>727</v>
-      </c>
-      <c r="C334" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D334" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E334" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F334" s="3" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A335" s="4">
-        <v>334</v>
-      </c>
-      <c r="B335" s="5" t="s">
-        <v>729</v>
-      </c>
-      <c r="C335" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D335" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E335" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F335" s="5" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A336" s="2">
-        <v>335</v>
-      </c>
-      <c r="B336" s="3" t="s">
-        <v>731</v>
-      </c>
-      <c r="C336" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D336" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E336" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F336" s="3" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A337" s="4">
-        <v>336</v>
-      </c>
-      <c r="B337" s="5" t="s">
-        <v>733</v>
-      </c>
-      <c r="C337" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D337" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E337" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F337" s="5" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A338" s="2">
-        <v>337</v>
-      </c>
-      <c r="B338" s="3" t="s">
-        <v>735</v>
-      </c>
-      <c r="C338" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D338" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E338" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F338" s="3" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A339" s="4">
-        <v>338</v>
-      </c>
-      <c r="B339" s="5" t="s">
-        <v>737</v>
-      </c>
-      <c r="C339" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D339" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E339" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F339" s="5" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A340" s="2">
-        <v>339</v>
-      </c>
-      <c r="B340" s="3" t="s">
-        <v>739</v>
-      </c>
-      <c r="C340" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D340" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E340" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F340" s="3" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A341" s="4">
-        <v>340</v>
-      </c>
-      <c r="B341" s="5" t="s">
-        <v>741</v>
-      </c>
-      <c r="C341" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D341" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E341" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F341" s="5" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A342" s="2">
-        <v>341</v>
-      </c>
-      <c r="B342" s="3" t="s">
-        <v>743</v>
-      </c>
-      <c r="C342" s="3" t="s">
-        <v>562</v>
-      </c>
-      <c r="D342" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E342" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F342" s="3" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A343" s="4">
-        <v>342</v>
-      </c>
-      <c r="B343" s="5" t="s">
-        <v>745</v>
-      </c>
-      <c r="C343" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="D343" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E343" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F343" s="5" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A344" s="2">
-        <v>343</v>
-      </c>
-      <c r="B344" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="C344" s="3" t="s">
-        <v>748</v>
-      </c>
-      <c r="D344" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E344" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F344" s="3" t="s">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A345" s="4">
-        <v>344</v>
-      </c>
-      <c r="B345" s="5" t="s">
-        <v>750</v>
-      </c>
-      <c r="C345" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="D345" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E345" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F345" s="5" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A346" s="2">
-        <v>345</v>
-      </c>
-      <c r="B346" s="3" t="s">
-        <v>752</v>
-      </c>
-      <c r="C346" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D346" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E346" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F346" s="3" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A347" s="4">
-        <v>346</v>
-      </c>
-      <c r="B347" s="5" t="s">
-        <v>754</v>
-      </c>
-      <c r="C347" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="D347" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E347" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F347" s="5" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A348" s="2">
-        <v>347</v>
-      </c>
-      <c r="B348" s="3" t="s">
-        <v>756</v>
-      </c>
-      <c r="C348" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D348" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E348" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F348" s="3" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A349" s="4">
-        <v>348</v>
-      </c>
-      <c r="B349" s="5" t="s">
-        <v>758</v>
-      </c>
-      <c r="C349" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D349" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E349" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F349" s="5" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A350" s="2">
-        <v>349</v>
-      </c>
-      <c r="B350" s="3" t="s">
-        <v>760</v>
-      </c>
-      <c r="C350" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D350" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E350" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F350" s="3" t="s">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A351" s="4">
-        <v>350</v>
-      </c>
-      <c r="B351" s="5" t="s">
-        <v>762</v>
-      </c>
-      <c r="C351" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="D351" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E351" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F351" s="5" t="s">
-        <v>763</v>
-      </c>
-    </row>
-    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A352" s="2">
-        <v>351</v>
-      </c>
-      <c r="B352" s="3" t="s">
-        <v>764</v>
-      </c>
-      <c r="C352" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D352" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E352" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F352" s="3" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A353" s="4">
-        <v>352</v>
-      </c>
-      <c r="B353" s="5" t="s">
-        <v>766</v>
-      </c>
-      <c r="C353" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D353" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E353" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F353" s="5" t="s">
-        <v>767</v>
-      </c>
-    </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A354" s="2">
-        <v>353</v>
-      </c>
-      <c r="B354" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="C354" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D354" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E354" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F354" s="3" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="355" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A355" s="4">
-        <v>354</v>
-      </c>
-      <c r="B355" s="5" t="s">
-        <v>770</v>
-      </c>
-      <c r="C355" s="5" t="s">
-        <v>771</v>
-      </c>
-      <c r="D355" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E355" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F355" s="5" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="356" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A356" s="2">
-        <v>355</v>
-      </c>
-      <c r="B356" s="3" t="s">
-        <v>773</v>
-      </c>
-      <c r="C356" s="3" t="s">
-        <v>771</v>
-      </c>
-      <c r="D356" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E356" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F356" s="3" t="s">
-        <v>774</v>
-      </c>
-    </row>
-    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A357" s="4">
-        <v>356</v>
-      </c>
-      <c r="B357" s="5" t="s">
-        <v>775</v>
-      </c>
-      <c r="C357" s="5" t="s">
-        <v>771</v>
-      </c>
-      <c r="D357" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E357" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F357" s="5" t="s">
-        <v>776</v>
-      </c>
-    </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A358" s="2">
-        <v>357</v>
-      </c>
-      <c r="B358" s="3" t="s">
-        <v>777</v>
-      </c>
-      <c r="C358" s="3" t="s">
-        <v>771</v>
-      </c>
-      <c r="D358" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E358" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F358" s="3" t="s">
-        <v>778</v>
-      </c>
-    </row>
-    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A359" s="4">
-        <v>358</v>
-      </c>
-      <c r="B359" s="5" t="s">
-        <v>779</v>
-      </c>
-      <c r="C359" s="5" t="s">
-        <v>780</v>
-      </c>
-      <c r="D359" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E359" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F359" s="5" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A360" s="2">
-        <v>359</v>
-      </c>
-      <c r="B360" s="3" t="s">
-        <v>782</v>
-      </c>
-      <c r="C360" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="D360" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E360" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F360" s="3" t="s">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A361" s="4">
-        <v>360</v>
-      </c>
-      <c r="B361" s="5" t="s">
-        <v>784</v>
-      </c>
-      <c r="C361" s="5" t="s">
-        <v>780</v>
-      </c>
-      <c r="D361" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E361" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F361" s="5" t="s">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A362" s="2">
-        <v>361</v>
-      </c>
-      <c r="B362" s="3" t="s">
-        <v>786</v>
-      </c>
-      <c r="C362" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="D362" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E362" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F362" s="3" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A363" s="4">
-        <v>362</v>
-      </c>
-      <c r="B363" s="5" t="s">
-        <v>788</v>
-      </c>
-      <c r="C363" s="5" t="s">
-        <v>780</v>
-      </c>
-      <c r="D363" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E363" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F363" s="5" t="s">
-        <v>789</v>
-      </c>
-    </row>
-    <row r="364" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A364" s="2">
-        <v>363</v>
-      </c>
-      <c r="B364" s="3" t="s">
-        <v>790</v>
-      </c>
-      <c r="C364" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="D364" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E364" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F364" s="3" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="365" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A365" s="4">
-        <v>364</v>
-      </c>
-      <c r="B365" s="5" t="s">
-        <v>792</v>
-      </c>
-      <c r="C365" s="5" t="s">
-        <v>793</v>
-      </c>
-      <c r="D365" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E365" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F365" s="5" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="366" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A366" s="2">
-        <v>365</v>
-      </c>
-      <c r="B366" s="3" t="s">
-        <v>795</v>
-      </c>
-      <c r="C366" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D366" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E366" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F366" s="3" t="s">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="367" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A367" s="4">
-        <v>366</v>
-      </c>
-      <c r="B367" s="5" t="s">
-        <v>797</v>
-      </c>
-      <c r="C367" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="D367" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E367" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F367" s="5" t="s">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="368" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A368" s="2">
-        <v>367</v>
-      </c>
-      <c r="B368" s="3" t="s">
-        <v>799</v>
-      </c>
-      <c r="C368" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D368" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E368" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F368" s="3" t="s">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A369" s="4">
-        <v>368</v>
-      </c>
-      <c r="B369" s="5" t="s">
-        <v>801</v>
-      </c>
-      <c r="C369" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="D369" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E369" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F369" s="5" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A370" s="2">
-        <v>369</v>
-      </c>
-      <c r="B370" s="3" t="s">
-        <v>803</v>
-      </c>
-      <c r="C370" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="D370" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E370" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F370" s="3" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A371" s="4">
-        <v>370</v>
-      </c>
-      <c r="B371" s="5" t="s">
-        <v>805</v>
-      </c>
-      <c r="C371" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="D371" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E371" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F371" s="5" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A372" s="2">
-        <v>371</v>
-      </c>
-      <c r="B372" s="3" t="s">
-        <v>807</v>
-      </c>
-      <c r="C372" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="D372" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E372" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F372" s="3" t="s">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A373" s="4">
-        <v>372</v>
-      </c>
-      <c r="B373" s="5" t="s">
-        <v>809</v>
-      </c>
-      <c r="C373" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="D373" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E373" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F373" s="5" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A374" s="2">
-        <v>373</v>
-      </c>
-      <c r="B374" s="3" t="s">
-        <v>811</v>
-      </c>
-      <c r="C374" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D374" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E374" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F374" s="3" t="s">
-        <v>812</v>
-      </c>
-    </row>
-    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A375" s="4">
-        <v>374</v>
-      </c>
-      <c r="B375" s="5" t="s">
-        <v>813</v>
-      </c>
-      <c r="C375" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="D375" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E375" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F375" s="5" t="s">
-        <v>814</v>
-      </c>
-    </row>
-    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A376" s="2">
-        <v>375</v>
-      </c>
-      <c r="B376" s="3" t="s">
-        <v>815</v>
-      </c>
-      <c r="C376" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D376" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E376" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F376" s="3" t="s">
-        <v>816</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Reapply "Add MTA descriptions and post-bind Risk ID assertions across tests"
This reverts commit 16604bb7a1af6699d627d6cd38b9ca1c68761085.
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="817">
   <si>
     <t>Run #</t>
   </si>
@@ -1580,6 +1580,888 @@
   </si>
   <si>
     <t>13/05/2026, 15:27:19</t>
+  </si>
+  <si>
+    <t>DA-MLI-537284133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:54:39</t>
+  </si>
+  <si>
+    <t>DA-MLI-537285133</t>
+  </si>
+  <si>
+    <t>13/05/2026, 15:56:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-080082134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 11:49:36</t>
+  </si>
+  <si>
+    <t>CP-MLI-062655134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 13:23:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-080091134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 13:48:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-080095134</t>
+  </si>
+  <si>
+    <t>TC_REG_042 | Cancel and reissue date today then MTA effective date cannot be yesterday</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:02:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-080099134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:07:56</t>
+  </si>
+  <si>
+    <t>DA-MLI-080102134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:14:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-080105134</t>
+  </si>
+  <si>
+    <t>TC_REG_043 | Create MTA then Cancel and Reissue then Create MTA</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:28:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-080112134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:40:30</t>
+  </si>
+  <si>
+    <t>DA-MLI-537294134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:52:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-537296134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 14:55:48</t>
+  </si>
+  <si>
+    <t>CP-MLI-062657134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:17:43</t>
+  </si>
+  <si>
+    <t>CP-MLI-062659134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:19:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-062679134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:24:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-062688134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:27:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-062705134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:30:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-080120134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 15:43:05</t>
+  </si>
+  <si>
+    <t>CP-NI-080127134</t>
+  </si>
+  <si>
+    <t>DT-MLIS-DF25.5.0 | CR-237340 |TC_34_S6_Verify Cancellation premiums are applied to the appropriate intermediary when user change the Intermediary Legal Entity on MTA _NB&gt;CRN&gt;MTA_Cancel the Policy Mid-term_NI commercial_Broker portal</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:19:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080129134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:23:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080132134</t>
+  </si>
+  <si>
+    <t>14/05/2026, 17:28:52</t>
+  </si>
+  <si>
+    <t>CP-NI-080495138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:32:40</t>
+  </si>
+  <si>
+    <t>CP-NI-080497138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:37:13</t>
+  </si>
+  <si>
+    <t>CP-NI-080499138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:41:41</t>
+  </si>
+  <si>
+    <t>CP-NI-080501138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:45:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080503138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:49:18</t>
+  </si>
+  <si>
+    <t>CP-NI-080506138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 08:53:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080510138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:02:42</t>
+  </si>
+  <si>
+    <t>CP-NI-080513138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:08:11</t>
+  </si>
+  <si>
+    <t>CP-NI-080516138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:12:55</t>
+  </si>
+  <si>
+    <t>CP-NI-080517138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:14:47</t>
+  </si>
+  <si>
+    <t>CP-NI-080520138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:21:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080523138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:26:08</t>
+  </si>
+  <si>
+    <t>CP-NI-080526138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:31:55</t>
+  </si>
+  <si>
+    <t>CP-NI-080528138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:37:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080532138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:46:06</t>
+  </si>
+  <si>
+    <t>CP-NI-080535138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 09:53:45</t>
+  </si>
+  <si>
+    <t>CP-NI-080538138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:02:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080541138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:09:12</t>
+  </si>
+  <si>
+    <t>CP-NI-080544138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:15:18</t>
+  </si>
+  <si>
+    <t>CP-NI-080547138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:20:19</t>
+  </si>
+  <si>
+    <t>CP-NI-080550138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:27:05</t>
+  </si>
+  <si>
+    <t>CP-NI-080553138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:32:16</t>
+  </si>
+  <si>
+    <t>CP-NI-080555138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:35:09</t>
+  </si>
+  <si>
+    <t>CP-NI-080558138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:41:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080561138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 10:51:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080564138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:00:13</t>
+  </si>
+  <si>
+    <t>CP-NI-062979138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:04:14</t>
+  </si>
+  <si>
+    <t>CP-NI-080567138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:17:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080570138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:22:21</t>
+  </si>
+  <si>
+    <t>CP-NI-080572138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:24:42</t>
+  </si>
+  <si>
+    <t>CP-NI-080575138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:29:27</t>
+  </si>
+  <si>
+    <t>CP-NI-080577138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:32:10</t>
+  </si>
+  <si>
+    <t>CP-NI-080580138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:38:36</t>
+  </si>
+  <si>
+    <t>CP-NI-080583138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:43:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080586138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:48:56</t>
+  </si>
+  <si>
+    <t>CP-NI-080589138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 11:55:02</t>
+  </si>
+  <si>
+    <t>CP-NI-080593138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:02:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080596138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:08:40</t>
+  </si>
+  <si>
+    <t>CP-NI-080599138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:14:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080602138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:21:46</t>
+  </si>
+  <si>
+    <t>CP-NI-080605138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:27:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080606138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:29:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080608138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 12:33:04</t>
+  </si>
+  <si>
+    <t>DA-MLI-080624138</t>
+  </si>
+  <si>
+    <t>TC_REG_045 | Source Submission -&gt; Change of Limit of Indemnity updates Limit of Indemnity after refresh</t>
+  </si>
+  <si>
+    <t>18/05/2026, 13:45:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-080626138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 13:51:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080628138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:00:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080672138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:11:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080717138</t>
+  </si>
+  <si>
+    <t>TC_REG_045 | Clear MTA flow on a live policy</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:25:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-080719138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:27:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-080722138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:29:04</t>
+  </si>
+  <si>
+    <t>DA-MLI-080726138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:33:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-080728138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:35:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-080729138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:38:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-080732138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:43:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-080735138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:46:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-080737138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:51:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-080738138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:52:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080741138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:55:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-080743138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 14:59:36</t>
+  </si>
+  <si>
+    <t>DA-MLI-080744138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:02:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-080745138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:04:44</t>
+  </si>
+  <si>
+    <t>DA-MLI-080747138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:09:36</t>
+  </si>
+  <si>
+    <t>DA-MLI-080750138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:14:18</t>
+  </si>
+  <si>
+    <t>DA-MLI-080753138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:20:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-080755138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:23:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-080759138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 15:29:58</t>
+  </si>
+  <si>
+    <t>DA-MLI-080769138</t>
+  </si>
+  <si>
+    <t>TC_REG_046 | Create MTA without bind, assert Insurance Policies (0) and Quotes (1), open Quote</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:17:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-080770138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:21:29</t>
+  </si>
+  <si>
+    <t>DA-MLI-080773138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:25:30</t>
+  </si>
+  <si>
+    <t>CP-NI-080776138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:35:28</t>
+  </si>
+  <si>
+    <t>CP-NI-080780138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:42:16</t>
+  </si>
+  <si>
+    <t>CP-NI-080783138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:48:31</t>
+  </si>
+  <si>
+    <t>CP-NI-080787138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:54:49</t>
+  </si>
+  <si>
+    <t>CP-NI-080789138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 16:57:11</t>
+  </si>
+  <si>
+    <t>CP-NI-080794138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:09:08</t>
+  </si>
+  <si>
+    <t>CP-NI-080798138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:15:09</t>
+  </si>
+  <si>
+    <t>CP-NI-063006138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 17:59:05</t>
+  </si>
+  <si>
+    <t>CP-NI-063005138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:00:36</t>
+  </si>
+  <si>
+    <t>CP-NI-080817138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:02:27</t>
+  </si>
+  <si>
+    <t>CP-NI-080823138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:07:26</t>
+  </si>
+  <si>
+    <t>CP-NI-080828138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:15:44</t>
+  </si>
+  <si>
+    <t>CP-NI-080835138</t>
+  </si>
+  <si>
+    <t>18/05/2026, 18:26:54</t>
+  </si>
+  <si>
+    <t>CP-NI-080956139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:10:46</t>
+  </si>
+  <si>
+    <t>CP-NI-080961139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:19:59</t>
+  </si>
+  <si>
+    <t>CP-NI-080969139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:32:28</t>
+  </si>
+  <si>
+    <t>CP-NI-080971139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:35:48</t>
+  </si>
+  <si>
+    <t>CP-NI-080973139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:38:51</t>
+  </si>
+  <si>
+    <t>CP-NI-080974139</t>
+  </si>
+  <si>
+    <t>19/05/2026, 15:40:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-063700140</t>
+  </si>
+  <si>
+    <t>TC_BDX_005_NB_MTA | Create NB-MTA (Mid-Term Adjustment) on a live policy</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:04:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-081093140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:06:43</t>
+  </si>
+  <si>
+    <t>DA-MLI-081094140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:10:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-081095140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:10:24</t>
+  </si>
+  <si>
+    <t>DA-MLI-081098140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 10:13:48</t>
+  </si>
+  <si>
+    <t>CP-MLI-081106140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:44:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-063836140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:50:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063843140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:55:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-063847140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:57:13</t>
+  </si>
+  <si>
+    <t>CP-MLI-063851140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:59:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-063852140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 12:59:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-081125140</t>
+  </si>
+  <si>
+    <t>TC_REG_047 | Save at quotes, verify SF related counts, resume and issue policy</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:37:39</t>
+  </si>
+  <si>
+    <t>DA-MLI-081127140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:46:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-081129140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 13:55:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-081130140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:01:19</t>
+  </si>
+  <si>
+    <t>DA-MLI-081133140</t>
+  </si>
+  <si>
+    <t>TC_REG_048 | NB-MTA validate Edit Terms Discount + Update Premium fallback and complete bind</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:43:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-081134140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:50:38</t>
+  </si>
+  <si>
+    <t>DA-MLI-081136140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 14:54:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-081138140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:00:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-081141140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:11:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-081143140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:21:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-081148140</t>
+  </si>
+  <si>
+    <t>TC_REG_049 | Create NB then update discount on Quotes tab and continue quote in Salesforce</t>
+  </si>
+  <si>
+    <t>20/05/2026, 15:46:33</t>
+  </si>
+  <si>
+    <t>DA-MLI-063952140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:50:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063954140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:53:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-063955140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:54:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-063956140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 17:59:42</t>
+  </si>
+  <si>
+    <t>DA-MLI-063967140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:40:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-063971140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:53:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-063974140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 18:59:59</t>
+  </si>
+  <si>
+    <t>DA-MLI-063977140</t>
+  </si>
+  <si>
+    <t>20/05/2026, 19:09:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-081322141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 15:55:11</t>
+  </si>
+  <si>
+    <t>DA-MLI-081332141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 16:00:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-081334141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 16:02:27</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F234"/>
+  <dimension ref="A1:F376"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -6704,6 +7586,2846 @@
         <v>522</v>
       </c>
     </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A235" s="4">
+        <v>234</v>
+      </c>
+      <c r="B235" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="C235" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D235" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E235" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F235" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A236" s="2">
+        <v>235</v>
+      </c>
+      <c r="B236" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D236" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E236" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F236" s="3" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A237" s="4">
+        <v>236</v>
+      </c>
+      <c r="B237" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="C237" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D237" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E237" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F237" s="5" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A238" s="2">
+        <v>237</v>
+      </c>
+      <c r="B238" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D238" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E238" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F238" s="3" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A239" s="4">
+        <v>238</v>
+      </c>
+      <c r="B239" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="C239" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E239" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F239" s="5" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A240" s="2">
+        <v>239</v>
+      </c>
+      <c r="B240" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D240" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E240" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F240" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A241" s="4">
+        <v>240</v>
+      </c>
+      <c r="B241" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="C241" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="D241" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E241" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F241" s="5" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A242" s="2">
+        <v>241</v>
+      </c>
+      <c r="B242" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="D242" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E242" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F242" s="3" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A243" s="4">
+        <v>242</v>
+      </c>
+      <c r="B243" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="C243" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="D243" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E243" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F243" s="5" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A244" s="2">
+        <v>243</v>
+      </c>
+      <c r="B244" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="D244" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E244" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F244" s="3" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A245" s="4">
+        <v>244</v>
+      </c>
+      <c r="B245" s="5" t="s">
+        <v>545</v>
+      </c>
+      <c r="C245" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D245" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E245" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F245" s="5" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A246" s="2">
+        <v>245</v>
+      </c>
+      <c r="B246" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D246" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E246" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A247" s="4">
+        <v>246</v>
+      </c>
+      <c r="B247" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C247" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E247" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F247" s="5" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A248" s="2">
+        <v>247</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D248" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E248" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F248" s="3" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A249" s="4">
+        <v>248</v>
+      </c>
+      <c r="B249" s="5" t="s">
+        <v>553</v>
+      </c>
+      <c r="C249" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E249" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F249" s="5" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A250" s="2">
+        <v>249</v>
+      </c>
+      <c r="B250" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D250" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E250" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F250" s="3" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A251" s="4">
+        <v>250</v>
+      </c>
+      <c r="B251" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="C251" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E251" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F251" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A252" s="2">
+        <v>251</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D252" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E252" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F252" s="3" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A253" s="4">
+        <v>252</v>
+      </c>
+      <c r="B253" s="5" t="s">
+        <v>561</v>
+      </c>
+      <c r="C253" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E253" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F253" s="5" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A254" s="2">
+        <v>253</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D254" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E254" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F254" s="3" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A255" s="4">
+        <v>254</v>
+      </c>
+      <c r="B255" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="C255" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E255" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F255" s="5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A256" s="2">
+        <v>255</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D256" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E256" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F256" s="3" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A257" s="4">
+        <v>256</v>
+      </c>
+      <c r="B257" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="C257" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E257" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F257" s="5" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A258" s="2">
+        <v>257</v>
+      </c>
+      <c r="B258" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D258" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E258" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F258" s="3" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A259" s="4">
+        <v>258</v>
+      </c>
+      <c r="B259" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="C259" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D259" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E259" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F259" s="5" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A260" s="2">
+        <v>259</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F260" s="3" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A261" s="4">
+        <v>260</v>
+      </c>
+      <c r="B261" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="C261" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E261" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F261" s="5" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A262" s="2">
+        <v>261</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F262" s="3" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A263" s="4">
+        <v>262</v>
+      </c>
+      <c r="B263" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="C263" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D263" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E263" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F263" s="5" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A264" s="2">
+        <v>263</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F264" s="3" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A265" s="4">
+        <v>264</v>
+      </c>
+      <c r="B265" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="C265" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D265" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E265" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F265" s="5" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A266" s="2">
+        <v>265</v>
+      </c>
+      <c r="B266" s="3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D266" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E266" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F266" s="3" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A267" s="4">
+        <v>266</v>
+      </c>
+      <c r="B267" s="5" t="s">
+        <v>590</v>
+      </c>
+      <c r="C267" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D267" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E267" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F267" s="5" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A268" s="2">
+        <v>267</v>
+      </c>
+      <c r="B268" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D268" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E268" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F268" s="3" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A269" s="4">
+        <v>268</v>
+      </c>
+      <c r="B269" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="C269" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D269" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E269" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F269" s="5" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A270" s="2">
+        <v>269</v>
+      </c>
+      <c r="B270" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D270" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E270" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F270" s="3" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A271" s="4">
+        <v>270</v>
+      </c>
+      <c r="B271" s="5" t="s">
+        <v>598</v>
+      </c>
+      <c r="C271" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D271" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E271" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F271" s="5" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A272" s="2">
+        <v>271</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D272" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E272" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F272" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A273" s="4">
+        <v>272</v>
+      </c>
+      <c r="B273" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="C273" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D273" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E273" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F273" s="5" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A274" s="2">
+        <v>273</v>
+      </c>
+      <c r="B274" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D274" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E274" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A275" s="4">
+        <v>274</v>
+      </c>
+      <c r="B275" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="C275" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D275" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E275" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F275" s="5" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A276" s="2">
+        <v>275</v>
+      </c>
+      <c r="B276" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E276" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F276" s="3" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A277" s="4">
+        <v>276</v>
+      </c>
+      <c r="B277" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="C277" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D277" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E277" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F277" s="5" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A278" s="2">
+        <v>277</v>
+      </c>
+      <c r="B278" s="3" t="s">
+        <v>612</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D278" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E278" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A279" s="4">
+        <v>278</v>
+      </c>
+      <c r="B279" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="C279" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D279" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E279" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F279" s="5" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A280" s="2">
+        <v>279</v>
+      </c>
+      <c r="B280" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D280" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E280" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A281" s="4">
+        <v>280</v>
+      </c>
+      <c r="B281" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="C281" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D281" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E281" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A282" s="2">
+        <v>281</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D282" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E282" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F282" s="3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A283" s="4">
+        <v>282</v>
+      </c>
+      <c r="B283" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="C283" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E283" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F283" s="5" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A284" s="2">
+        <v>283</v>
+      </c>
+      <c r="B284" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D284" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E284" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F284" s="3" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A285" s="4">
+        <v>284</v>
+      </c>
+      <c r="B285" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="C285" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D285" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E285" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F285" s="5" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A286" s="2">
+        <v>285</v>
+      </c>
+      <c r="B286" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D286" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E286" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F286" s="3" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A287" s="4">
+        <v>286</v>
+      </c>
+      <c r="B287" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="C287" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E287" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F287" s="5" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A288" s="2">
+        <v>287</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E288" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F288" s="3" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A289" s="4">
+        <v>288</v>
+      </c>
+      <c r="B289" s="5" t="s">
+        <v>634</v>
+      </c>
+      <c r="C289" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D289" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E289" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F289" s="5" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A290" s="2">
+        <v>289</v>
+      </c>
+      <c r="B290" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D290" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E290" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F290" s="3" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A291" s="4">
+        <v>290</v>
+      </c>
+      <c r="B291" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="C291" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D291" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E291" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F291" s="5" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A292" s="2">
+        <v>291</v>
+      </c>
+      <c r="B292" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A293" s="4">
+        <v>292</v>
+      </c>
+      <c r="B293" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="C293" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E293" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F293" s="5" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A294" s="2">
+        <v>293</v>
+      </c>
+      <c r="B294" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A295" s="4">
+        <v>294</v>
+      </c>
+      <c r="B295" s="5" t="s">
+        <v>646</v>
+      </c>
+      <c r="C295" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E295" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F295" s="5" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A296" s="2">
+        <v>295</v>
+      </c>
+      <c r="B296" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F296" s="3" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A297" s="4">
+        <v>296</v>
+      </c>
+      <c r="B297" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="C297" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D297" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E297" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F297" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A298" s="2">
+        <v>297</v>
+      </c>
+      <c r="B298" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F298" s="3" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A299" s="4">
+        <v>298</v>
+      </c>
+      <c r="B299" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="C299" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="D299" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E299" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F299" s="5" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A300" s="2">
+        <v>299</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A301" s="4">
+        <v>300</v>
+      </c>
+      <c r="B301" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="C301" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="D301" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E301" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F301" s="5" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A302" s="2">
+        <v>301</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A303" s="4">
+        <v>302</v>
+      </c>
+      <c r="B303" s="5" t="s">
+        <v>663</v>
+      </c>
+      <c r="C303" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E303" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F303" s="5" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A304" s="2">
+        <v>303</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A305" s="4">
+        <v>304</v>
+      </c>
+      <c r="B305" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="C305" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D305" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E305" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F305" s="5" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A306" s="2">
+        <v>305</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F306" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A307" s="4">
+        <v>306</v>
+      </c>
+      <c r="B307" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="C307" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D307" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E307" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F307" s="5" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A308" s="2">
+        <v>307</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>674</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F308" s="3" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A309" s="4">
+        <v>308</v>
+      </c>
+      <c r="B309" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="C309" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D309" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E309" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F309" s="5" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A310" s="2">
+        <v>309</v>
+      </c>
+      <c r="B310" s="3" t="s">
+        <v>678</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F310" s="3" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A311" s="4">
+        <v>310</v>
+      </c>
+      <c r="B311" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="C311" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D311" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E311" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F311" s="5" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A312" s="2">
+        <v>311</v>
+      </c>
+      <c r="B312" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F312" s="3" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A313" s="4">
+        <v>312</v>
+      </c>
+      <c r="B313" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="C313" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D313" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E313" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F313" s="5" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A314" s="2">
+        <v>313</v>
+      </c>
+      <c r="B314" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D314" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E314" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F314" s="3" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A315" s="4">
+        <v>314</v>
+      </c>
+      <c r="B315" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="C315" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D315" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E315" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F315" s="5" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A316" s="2">
+        <v>315</v>
+      </c>
+      <c r="B316" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D316" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E316" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F316" s="3" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A317" s="4">
+        <v>316</v>
+      </c>
+      <c r="B317" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="C317" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D317" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E317" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F317" s="5" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A318" s="2">
+        <v>317</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D318" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E318" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F318" s="3" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A319" s="4">
+        <v>318</v>
+      </c>
+      <c r="B319" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="C319" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D319" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E319" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F319" s="5" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A320" s="2">
+        <v>319</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D320" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E320" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F320" s="3" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321" s="4">
+        <v>320</v>
+      </c>
+      <c r="B321" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="C321" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="D321" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E321" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F321" s="5" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A322" s="2">
+        <v>321</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="C322" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D322" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E322" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F322" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A323" s="4">
+        <v>322</v>
+      </c>
+      <c r="B323" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="C323" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="D323" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E323" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F323" s="5" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A324" s="2">
+        <v>323</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="C324" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="D324" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E324" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F324" s="3" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A325" s="4">
+        <v>324</v>
+      </c>
+      <c r="B325" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="C325" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D325" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E325" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F325" s="5" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A326" s="2">
+        <v>325</v>
+      </c>
+      <c r="B326" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="C326" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D326" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E326" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F326" s="3" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A327" s="4">
+        <v>326</v>
+      </c>
+      <c r="B327" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="C327" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D327" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E327" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F327" s="5" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A328" s="2">
+        <v>327</v>
+      </c>
+      <c r="B328" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="C328" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D328" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E328" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F328" s="3" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A329" s="4">
+        <v>328</v>
+      </c>
+      <c r="B329" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="C329" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D329" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E329" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F329" s="5" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A330" s="2">
+        <v>329</v>
+      </c>
+      <c r="B330" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="C330" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D330" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E330" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F330" s="3" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A331" s="4">
+        <v>330</v>
+      </c>
+      <c r="B331" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="C331" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D331" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E331" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F331" s="5" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A332" s="2">
+        <v>331</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="C332" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D332" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E332" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F332" s="3" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A333" s="4">
+        <v>332</v>
+      </c>
+      <c r="B333" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="C333" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D333" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E333" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F333" s="5" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A334" s="2">
+        <v>333</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>727</v>
+      </c>
+      <c r="C334" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D334" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E334" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F334" s="3" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A335" s="4">
+        <v>334</v>
+      </c>
+      <c r="B335" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="C335" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D335" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E335" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F335" s="5" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A336" s="2">
+        <v>335</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="C336" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D336" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E336" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F336" s="3" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A337" s="4">
+        <v>336</v>
+      </c>
+      <c r="B337" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="C337" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D337" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E337" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F337" s="5" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A338" s="2">
+        <v>337</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="C338" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D338" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E338" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F338" s="3" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A339" s="4">
+        <v>338</v>
+      </c>
+      <c r="B339" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="C339" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D339" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E339" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F339" s="5" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A340" s="2">
+        <v>339</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>739</v>
+      </c>
+      <c r="C340" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D340" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E340" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F340" s="3" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A341" s="4">
+        <v>340</v>
+      </c>
+      <c r="B341" s="5" t="s">
+        <v>741</v>
+      </c>
+      <c r="C341" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D341" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E341" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F341" s="5" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A342" s="2">
+        <v>341</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>743</v>
+      </c>
+      <c r="C342" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D342" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E342" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F342" s="3" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A343" s="4">
+        <v>342</v>
+      </c>
+      <c r="B343" s="5" t="s">
+        <v>745</v>
+      </c>
+      <c r="C343" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D343" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E343" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F343" s="5" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A344" s="2">
+        <v>343</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="C344" s="3" t="s">
+        <v>748</v>
+      </c>
+      <c r="D344" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E344" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F344" s="3" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A345" s="4">
+        <v>344</v>
+      </c>
+      <c r="B345" s="5" t="s">
+        <v>750</v>
+      </c>
+      <c r="C345" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D345" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E345" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F345" s="5" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A346" s="2">
+        <v>345</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>752</v>
+      </c>
+      <c r="C346" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D346" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E346" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F346" s="3" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A347" s="4">
+        <v>346</v>
+      </c>
+      <c r="B347" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="C347" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D347" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E347" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F347" s="5" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A348" s="2">
+        <v>347</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="C348" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D348" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E348" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F348" s="3" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A349" s="4">
+        <v>348</v>
+      </c>
+      <c r="B349" s="5" t="s">
+        <v>758</v>
+      </c>
+      <c r="C349" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D349" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E349" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F349" s="5" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A350" s="2">
+        <v>349</v>
+      </c>
+      <c r="B350" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="C350" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D350" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E350" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F350" s="3" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A351" s="4">
+        <v>350</v>
+      </c>
+      <c r="B351" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="C351" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D351" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E351" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F351" s="5" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A352" s="2">
+        <v>351</v>
+      </c>
+      <c r="B352" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="C352" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D352" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E352" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F352" s="3" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A353" s="4">
+        <v>352</v>
+      </c>
+      <c r="B353" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="C353" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D353" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E353" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F353" s="5" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A354" s="2">
+        <v>353</v>
+      </c>
+      <c r="B354" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E354" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F354" s="3" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="355" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A355" s="4">
+        <v>354</v>
+      </c>
+      <c r="B355" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="C355" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="D355" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E355" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F355" s="5" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="356" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A356" s="2">
+        <v>355</v>
+      </c>
+      <c r="B356" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E356" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F356" s="3" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A357" s="4">
+        <v>356</v>
+      </c>
+      <c r="B357" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="C357" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="D357" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E357" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F357" s="5" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A358" s="2">
+        <v>357</v>
+      </c>
+      <c r="B358" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E358" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F358" s="3" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A359" s="4">
+        <v>358</v>
+      </c>
+      <c r="B359" s="5" t="s">
+        <v>779</v>
+      </c>
+      <c r="C359" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D359" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E359" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F359" s="5" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A360" s="2">
+        <v>359</v>
+      </c>
+      <c r="B360" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E360" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F360" s="3" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A361" s="4">
+        <v>360</v>
+      </c>
+      <c r="B361" s="5" t="s">
+        <v>784</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D361" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E361" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F361" s="5" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A362" s="2">
+        <v>361</v>
+      </c>
+      <c r="B362" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C362" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E362" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F362" s="3" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A363" s="4">
+        <v>362</v>
+      </c>
+      <c r="B363" s="5" t="s">
+        <v>788</v>
+      </c>
+      <c r="C363" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D363" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E363" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F363" s="5" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="364" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A364" s="2">
+        <v>363</v>
+      </c>
+      <c r="B364" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F364" s="3" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="365" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A365" s="4">
+        <v>364</v>
+      </c>
+      <c r="B365" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="C365" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="D365" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E365" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F365" s="5" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="366" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A366" s="2">
+        <v>365</v>
+      </c>
+      <c r="B366" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="C366" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D366" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E366" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F366" s="3" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="367" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A367" s="4">
+        <v>366</v>
+      </c>
+      <c r="B367" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="C367" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D367" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E367" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F367" s="5" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="368" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A368" s="2">
+        <v>367</v>
+      </c>
+      <c r="B368" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="C368" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D368" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E368" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F368" s="3" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A369" s="4">
+        <v>368</v>
+      </c>
+      <c r="B369" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D369" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E369" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F369" s="5" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A370" s="2">
+        <v>369</v>
+      </c>
+      <c r="B370" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="C370" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D370" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E370" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F370" s="3" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A371" s="4">
+        <v>370</v>
+      </c>
+      <c r="B371" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="C371" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D371" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E371" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F371" s="5" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A372" s="2">
+        <v>371</v>
+      </c>
+      <c r="B372" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="C372" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D372" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E372" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F372" s="3" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A373" s="4">
+        <v>372</v>
+      </c>
+      <c r="B373" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="C373" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D373" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E373" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F373" s="5" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A374" s="2">
+        <v>373</v>
+      </c>
+      <c r="B374" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="C374" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D374" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E374" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F374" s="3" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A375" s="4">
+        <v>374</v>
+      </c>
+      <c r="B375" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="C375" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D375" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E375" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F375" s="5" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A376" s="2">
+        <v>375</v>
+      </c>
+      <c r="B376" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="C376" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D376" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E376" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F376" s="3" t="s">
+        <v>816</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
chore: update regression tests and dashboard generation
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1901" uniqueCount="825">
   <si>
     <t>Run #</t>
   </si>
@@ -2462,6 +2462,30 @@
   </si>
   <si>
     <t>21/05/2026, 16:02:27</t>
+  </si>
+  <si>
+    <t>DA-MLI-081348141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 17:02:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-064567141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 17:09:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-081353141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 17:14:20</t>
+  </si>
+  <si>
+    <t>DA-MLI-081355141</t>
+  </si>
+  <si>
+    <t>21/05/2026, 17:19:08</t>
   </si>
 </sst>
 </file>
@@ -2895,7 +2919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F376"/>
+  <dimension ref="A1:F380"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -10426,6 +10450,86 @@
         <v>816</v>
       </c>
     </row>
+    <row r="377" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A377" s="4">
+        <v>376</v>
+      </c>
+      <c r="B377" s="5" t="s">
+        <v>817</v>
+      </c>
+      <c r="C377" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D377" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E377" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F377" s="5" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="378" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A378" s="2">
+        <v>377</v>
+      </c>
+      <c r="B378" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="C378" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D378" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E378" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F378" s="3" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="379" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A379" s="4">
+        <v>378</v>
+      </c>
+      <c r="B379" s="5" t="s">
+        <v>821</v>
+      </c>
+      <c r="C379" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D379" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E379" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F379" s="5" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="380" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A380" s="2">
+        <v>379</v>
+      </c>
+      <c r="B380" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="C380" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="D380" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E380" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F380" s="3" t="s">
+        <v>824</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
chore: update tests, salesforce flow, and dashboard artifacts
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1901" uniqueCount="825">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="1012">
   <si>
     <t>Run #</t>
   </si>
@@ -2486,6 +2486,567 @@
   </si>
   <si>
     <t>21/05/2026, 17:19:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-065037142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:03:41</t>
+  </si>
+  <si>
+    <t>DA-MLI-065038142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:07:23</t>
+  </si>
+  <si>
+    <t>DA-MLI-065039142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:14:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-065040142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:16:28</t>
+  </si>
+  <si>
+    <t>DA-MLI-065043142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:20:43</t>
+  </si>
+  <si>
+    <t>DA-MLI-065048142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:23:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-065051142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:24:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-065053142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:25:25</t>
+  </si>
+  <si>
+    <t>DA-MLI-065054142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:25:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-065062142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:28:40</t>
+  </si>
+  <si>
+    <t>DA-MLI-065066142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:30:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-065067142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:31:48</t>
+  </si>
+  <si>
+    <t>DA-MLI-065068142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:32:20</t>
+  </si>
+  <si>
+    <t>DA-MLI-065071142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:36:39</t>
+  </si>
+  <si>
+    <t>DA-MLI-065074142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:43:33</t>
+  </si>
+  <si>
+    <t>CP-MLI-081502142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:53:10</t>
+  </si>
+  <si>
+    <t>CP-MLI-081504142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 15:54:35</t>
+  </si>
+  <si>
+    <t>DA-MLI-081509142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:00:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-081510142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:02:38</t>
+  </si>
+  <si>
+    <t>CP-NI-081514142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:08:10</t>
+  </si>
+  <si>
+    <t>CP-NI-081515142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:08:56</t>
+  </si>
+  <si>
+    <t>CP-SC-081516142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:09:47</t>
+  </si>
+  <si>
+    <t>CP-SC-081518142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:10:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-081519142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:11:18</t>
+  </si>
+  <si>
+    <t>DA-MLI-081521142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:12:05</t>
+  </si>
+  <si>
+    <t>DA-NI-081522142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:12:56</t>
+  </si>
+  <si>
+    <t>DA-NI-081523142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:13:45</t>
+  </si>
+  <si>
+    <t>DA-SC-081525142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:14:34</t>
+  </si>
+  <si>
+    <t>DA-SC-081526142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:15:24</t>
+  </si>
+  <si>
+    <t>DA-MLI-081527142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:16:08</t>
+  </si>
+  <si>
+    <t>CP-MLI-081532142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:17:11</t>
+  </si>
+  <si>
+    <t>CP-SC-081533142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:18:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-081534142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:19:34</t>
+  </si>
+  <si>
+    <t>DA-MLI-081537142</t>
+  </si>
+  <si>
+    <t>22/05/2026, 16:21:43</t>
+  </si>
+  <si>
+    <t>CP-NI-081858145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 14:52:13</t>
+  </si>
+  <si>
+    <t>CP-NI-081859145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:00:32</t>
+  </si>
+  <si>
+    <t>CP-NI-081862145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:06:53</t>
+  </si>
+  <si>
+    <t>CP-NI-081865145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:22:30</t>
+  </si>
+  <si>
+    <t>CP-NI-081868145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:31:18</t>
+  </si>
+  <si>
+    <t>CP-NI-081871145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:42:26</t>
+  </si>
+  <si>
+    <t>CP-NI-081874145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:47:07</t>
+  </si>
+  <si>
+    <t>CP-NI-081877145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 15:52:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-066605145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:04:10</t>
+  </si>
+  <si>
+    <t>CP-MLI-066607145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:08:59</t>
+  </si>
+  <si>
+    <t>CP-MLI-066609145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:10:23</t>
+  </si>
+  <si>
+    <t>DA-MLI-066614145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:16:44</t>
+  </si>
+  <si>
+    <t>DA-MLI-066615145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:19:12</t>
+  </si>
+  <si>
+    <t>CP-NI-066616145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 17:28:33</t>
+  </si>
+  <si>
+    <t>CP-MLI-537344145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 20:54:55</t>
+  </si>
+  <si>
+    <t>CP-MLI-537346145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 20:56:14</t>
+  </si>
+  <si>
+    <t>DA-MLI-537348145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 20:57:22</t>
+  </si>
+  <si>
+    <t>DA-MLI-537349145</t>
+  </si>
+  <si>
+    <t>25/05/2026, 20:59:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-537351145</t>
+  </si>
+  <si>
+    <t>TC_SAN_015 | Create MTA (Mid-Term Adjustment) on a live policy</t>
+  </si>
+  <si>
+    <t>25/05/2026, 21:08:05</t>
+  </si>
+  <si>
+    <t>DA-MLI-537353145</t>
+  </si>
+  <si>
+    <t>TC_SAN_016 | Cancel and reissue a live policy</t>
+  </si>
+  <si>
+    <t>25/05/2026, 21:12:22</t>
+  </si>
+  <si>
+    <t>CP-MLI-057893146</t>
+  </si>
+  <si>
+    <t>SIT1</t>
+  </si>
+  <si>
+    <t>26/05/2026, 19:22:47</t>
+  </si>
+  <si>
+    <t>DA-MLI-057894146</t>
+  </si>
+  <si>
+    <t>26/05/2026, 19:25:18</t>
+  </si>
+  <si>
+    <t>DA-MLI-057895146</t>
+  </si>
+  <si>
+    <t>26/05/2026, 19:27:40</t>
+  </si>
+  <si>
+    <t>CP-NI-082181147</t>
+  </si>
+  <si>
+    <t>DT-MLIS-DF25.5.0 | CR-237340 | TC_34_S6_Verify Cancellation premiums are applied to the appropriate intermediary when user change the Intermediary Legal Entity on MTA _NB&gt;MTA&gt;Cancel the Policy from Inception_NI commercial_Broker portal</t>
+  </si>
+  <si>
+    <t>27/05/2026, 14:04:39</t>
+  </si>
+  <si>
+    <t>CP-NI-082183147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 14:19:01</t>
+  </si>
+  <si>
+    <t>CP-NI-082185147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 14:32:14</t>
+  </si>
+  <si>
+    <t>CP-NI-082187147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 14:41:23</t>
+  </si>
+  <si>
+    <t>CP-NI-082190147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 14:50:18</t>
+  </si>
+  <si>
+    <t>CP-NI-082196147</t>
+  </si>
+  <si>
+    <t>DT-MLIS-DF25.5.0 | CR-237340 | TC_34_S6_NB&gt;MTA_Negative MTA Premium should not allow Bind_NI commercial_Broker portal</t>
+  </si>
+  <si>
+    <t>27/05/2026, 15:08:03</t>
+  </si>
+  <si>
+    <t>CP-NI-082199147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 15:20:12</t>
+  </si>
+  <si>
+    <t>CP-NI-082200147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 15:22:25</t>
+  </si>
+  <si>
+    <t>CP-NI-082202147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 15:27:21</t>
+  </si>
+  <si>
+    <t>CP-NI-082203147</t>
+  </si>
+  <si>
+    <t>27/05/2026, 15:30:30</t>
+  </si>
+  <si>
+    <t>CP-MLI-082815153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:11:18</t>
+  </si>
+  <si>
+    <t>CP-MLI-082817153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:12:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-082822153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:19:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-082823153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:21:45</t>
+  </si>
+  <si>
+    <t>DA-MLI-082824153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:23:09</t>
+  </si>
+  <si>
+    <t>DA-MLI-082828153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:24:30</t>
+  </si>
+  <si>
+    <t>DA-MLI-082829153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:27:44</t>
+  </si>
+  <si>
+    <t>DA-MLI-082831153</t>
+  </si>
+  <si>
+    <t>02/06/2026, 21:31:09</t>
+  </si>
+  <si>
+    <t>CP-NI-083561154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:21:59</t>
+  </si>
+  <si>
+    <t>CP-NI-083564154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:22:41</t>
+  </si>
+  <si>
+    <t>CP-SC-083569154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:23:24</t>
+  </si>
+  <si>
+    <t>CP-SC-083572154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:24:06</t>
+  </si>
+  <si>
+    <t>DA-MLI-083576154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:24:47</t>
+  </si>
+  <si>
+    <t>DA-MLI-083581154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:25:25</t>
+  </si>
+  <si>
+    <t>DA-NI-083589154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:26:10</t>
+  </si>
+  <si>
+    <t>DA-NI-083591154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:26:52</t>
+  </si>
+  <si>
+    <t>DA-SC-083602154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:27:34</t>
+  </si>
+  <si>
+    <t>DA-SC-083606154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:28:13</t>
+  </si>
+  <si>
+    <t>DA-MLI-083610154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:28:47</t>
+  </si>
+  <si>
+    <t>CP-MLI-083617154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:29:44</t>
+  </si>
+  <si>
+    <t>CP-SC-083625154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:31:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-083630154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:32:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-083642154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:34:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-083668154</t>
+  </si>
+  <si>
+    <t>03/06/2026, 21:38:34</t>
   </si>
 </sst>
 </file>
@@ -2919,7 +3480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F380"/>
+  <dimension ref="A1:F471"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -10530,6 +11091,1826 @@
         <v>824</v>
       </c>
     </row>
+    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A381" s="4">
+        <v>380</v>
+      </c>
+      <c r="B381" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="C381" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D381" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E381" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F381" s="5" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A382" s="2">
+        <v>381</v>
+      </c>
+      <c r="B382" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="C382" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D382" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E382" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F382" s="3" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A383" s="4">
+        <v>382</v>
+      </c>
+      <c r="B383" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C383" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D383" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E383" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F383" s="5" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A384" s="2">
+        <v>383</v>
+      </c>
+      <c r="B384" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="C384" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D384" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E384" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F384" s="3" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="385" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A385" s="4">
+        <v>384</v>
+      </c>
+      <c r="B385" s="5" t="s">
+        <v>833</v>
+      </c>
+      <c r="C385" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D385" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E385" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F385" s="5" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="386" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A386" s="2">
+        <v>385</v>
+      </c>
+      <c r="B386" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="C386" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D386" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E386" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F386" s="3" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="387" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A387" s="4">
+        <v>386</v>
+      </c>
+      <c r="B387" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="C387" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D387" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E387" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F387" s="5" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="388" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A388" s="2">
+        <v>387</v>
+      </c>
+      <c r="B388" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="C388" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D388" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E388" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F388" s="3" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="389" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A389" s="4">
+        <v>388</v>
+      </c>
+      <c r="B389" s="5" t="s">
+        <v>841</v>
+      </c>
+      <c r="C389" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D389" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E389" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F389" s="5" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="390" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A390" s="2">
+        <v>389</v>
+      </c>
+      <c r="B390" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="C390" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D390" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E390" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F390" s="3" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="391" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A391" s="4">
+        <v>390</v>
+      </c>
+      <c r="B391" s="5" t="s">
+        <v>845</v>
+      </c>
+      <c r="C391" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D391" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E391" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F391" s="5" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="392" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A392" s="2">
+        <v>391</v>
+      </c>
+      <c r="B392" s="3" t="s">
+        <v>847</v>
+      </c>
+      <c r="C392" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D392" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E392" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F392" s="3" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="393" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A393" s="4">
+        <v>392</v>
+      </c>
+      <c r="B393" s="5" t="s">
+        <v>849</v>
+      </c>
+      <c r="C393" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="D393" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E393" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F393" s="5" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="394" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A394" s="2">
+        <v>393</v>
+      </c>
+      <c r="B394" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="C394" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D394" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E394" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F394" s="3" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="395" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A395" s="4">
+        <v>394</v>
+      </c>
+      <c r="B395" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="C395" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D395" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E395" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F395" s="5" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="396" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A396" s="2">
+        <v>395</v>
+      </c>
+      <c r="B396" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="C396" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D396" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E396" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F396" s="3" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="397" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A397" s="4">
+        <v>396</v>
+      </c>
+      <c r="B397" s="5" t="s">
+        <v>857</v>
+      </c>
+      <c r="C397" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D397" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E397" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F397" s="5" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="398" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A398" s="2">
+        <v>397</v>
+      </c>
+      <c r="B398" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D398" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E398" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F398" s="3" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="399" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A399" s="4">
+        <v>398</v>
+      </c>
+      <c r="B399" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="C399" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D399" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E399" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F399" s="5" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="400" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A400" s="2">
+        <v>399</v>
+      </c>
+      <c r="B400" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D400" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E400" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F400" s="3" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="401" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A401" s="4">
+        <v>400</v>
+      </c>
+      <c r="B401" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="C401" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D401" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E401" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F401" s="5" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="402" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A402" s="2">
+        <v>401</v>
+      </c>
+      <c r="B402" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="C402" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D402" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E402" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F402" s="3" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="403" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A403" s="4">
+        <v>402</v>
+      </c>
+      <c r="B403" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="C403" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D403" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E403" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F403" s="5" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="404" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A404" s="2">
+        <v>403</v>
+      </c>
+      <c r="B404" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="C404" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D404" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E404" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F404" s="3" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="405" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A405" s="4">
+        <v>404</v>
+      </c>
+      <c r="B405" s="5" t="s">
+        <v>873</v>
+      </c>
+      <c r="C405" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D405" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E405" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F405" s="5" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="406" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A406" s="2">
+        <v>405</v>
+      </c>
+      <c r="B406" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="C406" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D406" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E406" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F406" s="3" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="407" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A407" s="4">
+        <v>406</v>
+      </c>
+      <c r="B407" s="5" t="s">
+        <v>877</v>
+      </c>
+      <c r="C407" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D407" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E407" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F407" s="5" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="408" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A408" s="2">
+        <v>407</v>
+      </c>
+      <c r="B408" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="C408" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D408" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E408" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F408" s="3" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="409" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A409" s="4">
+        <v>408</v>
+      </c>
+      <c r="B409" s="5" t="s">
+        <v>881</v>
+      </c>
+      <c r="C409" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D409" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E409" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F409" s="5" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="410" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A410" s="2">
+        <v>409</v>
+      </c>
+      <c r="B410" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="C410" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D410" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E410" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F410" s="3" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="411" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A411" s="4">
+        <v>410</v>
+      </c>
+      <c r="B411" s="5" t="s">
+        <v>885</v>
+      </c>
+      <c r="C411" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D411" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E411" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F411" s="5" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="412" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A412" s="2">
+        <v>411</v>
+      </c>
+      <c r="B412" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="C412" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D412" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E412" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F412" s="3" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="413" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A413" s="4">
+        <v>412</v>
+      </c>
+      <c r="B413" s="5" t="s">
+        <v>889</v>
+      </c>
+      <c r="C413" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D413" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E413" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F413" s="5" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="414" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A414" s="2">
+        <v>413</v>
+      </c>
+      <c r="B414" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="C414" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D414" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E414" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F414" s="3" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="415" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A415" s="4">
+        <v>414</v>
+      </c>
+      <c r="B415" s="5" t="s">
+        <v>893</v>
+      </c>
+      <c r="C415" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D415" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E415" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F415" s="5" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="416" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A416" s="2">
+        <v>415</v>
+      </c>
+      <c r="B416" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="C416" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D416" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E416" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F416" s="3" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="417" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A417" s="4">
+        <v>416</v>
+      </c>
+      <c r="B417" s="5" t="s">
+        <v>897</v>
+      </c>
+      <c r="C417" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D417" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E417" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F417" s="5" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="418" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A418" s="2">
+        <v>417</v>
+      </c>
+      <c r="B418" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="C418" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D418" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E418" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F418" s="3" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="419" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A419" s="4">
+        <v>418</v>
+      </c>
+      <c r="B419" s="5" t="s">
+        <v>901</v>
+      </c>
+      <c r="C419" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D419" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E419" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F419" s="5" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="420" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A420" s="2">
+        <v>419</v>
+      </c>
+      <c r="B420" s="3" t="s">
+        <v>903</v>
+      </c>
+      <c r="C420" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D420" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E420" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F420" s="3" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="421" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A421" s="4">
+        <v>420</v>
+      </c>
+      <c r="B421" s="5" t="s">
+        <v>905</v>
+      </c>
+      <c r="C421" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D421" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E421" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F421" s="5" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="422" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A422" s="2">
+        <v>421</v>
+      </c>
+      <c r="B422" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="C422" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D422" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E422" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F422" s="3" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="423" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A423" s="4">
+        <v>422</v>
+      </c>
+      <c r="B423" s="5" t="s">
+        <v>909</v>
+      </c>
+      <c r="C423" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D423" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E423" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F423" s="5" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="424" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A424" s="2">
+        <v>423</v>
+      </c>
+      <c r="B424" s="3" t="s">
+        <v>911</v>
+      </c>
+      <c r="C424" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D424" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E424" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F424" s="3" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="425" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A425" s="4">
+        <v>424</v>
+      </c>
+      <c r="B425" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="C425" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D425" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E425" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F425" s="5" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="426" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A426" s="2">
+        <v>425</v>
+      </c>
+      <c r="B426" s="3" t="s">
+        <v>915</v>
+      </c>
+      <c r="C426" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D426" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E426" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F426" s="3" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="427" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A427" s="4">
+        <v>426</v>
+      </c>
+      <c r="B427" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="C427" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D427" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E427" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F427" s="5" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="428" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A428" s="2">
+        <v>427</v>
+      </c>
+      <c r="B428" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="C428" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="D428" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E428" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F428" s="3" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="429" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A429" s="4">
+        <v>428</v>
+      </c>
+      <c r="B429" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="C429" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D429" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E429" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F429" s="5" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="430" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A430" s="2">
+        <v>429</v>
+      </c>
+      <c r="B430" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="C430" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D430" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E430" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F430" s="3" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="431" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A431" s="4">
+        <v>430</v>
+      </c>
+      <c r="B431" s="5" t="s">
+        <v>925</v>
+      </c>
+      <c r="C431" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D431" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E431" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F431" s="5" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="432" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A432" s="2">
+        <v>431</v>
+      </c>
+      <c r="B432" s="3" t="s">
+        <v>927</v>
+      </c>
+      <c r="C432" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D432" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E432" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F432" s="3" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="433" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A433" s="4">
+        <v>432</v>
+      </c>
+      <c r="B433" s="5" t="s">
+        <v>929</v>
+      </c>
+      <c r="C433" s="5" t="s">
+        <v>930</v>
+      </c>
+      <c r="D433" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E433" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F433" s="5" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="434" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A434" s="2">
+        <v>433</v>
+      </c>
+      <c r="B434" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="C434" s="3" t="s">
+        <v>933</v>
+      </c>
+      <c r="D434" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E434" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F434" s="3" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="435" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A435" s="4">
+        <v>434</v>
+      </c>
+      <c r="B435" s="5" t="s">
+        <v>935</v>
+      </c>
+      <c r="C435" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D435" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E435" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F435" s="5" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="436" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A436" s="2">
+        <v>435</v>
+      </c>
+      <c r="B436" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="C436" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D436" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E436" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F436" s="3" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="437" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A437" s="4">
+        <v>436</v>
+      </c>
+      <c r="B437" s="5" t="s">
+        <v>940</v>
+      </c>
+      <c r="C437" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D437" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E437" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F437" s="5" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="438" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A438" s="2">
+        <v>437</v>
+      </c>
+      <c r="B438" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="C438" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="D438" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E438" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F438" s="3" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="439" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A439" s="4">
+        <v>438</v>
+      </c>
+      <c r="B439" s="5" t="s">
+        <v>945</v>
+      </c>
+      <c r="C439" s="5" t="s">
+        <v>943</v>
+      </c>
+      <c r="D439" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E439" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F439" s="5" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="440" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A440" s="2">
+        <v>439</v>
+      </c>
+      <c r="B440" s="3" t="s">
+        <v>947</v>
+      </c>
+      <c r="C440" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="D440" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E440" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F440" s="3" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="441" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A441" s="4">
+        <v>440</v>
+      </c>
+      <c r="B441" s="5" t="s">
+        <v>949</v>
+      </c>
+      <c r="C441" s="5" t="s">
+        <v>943</v>
+      </c>
+      <c r="D441" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E441" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F441" s="5" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="442" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A442" s="2">
+        <v>441</v>
+      </c>
+      <c r="B442" s="3" t="s">
+        <v>951</v>
+      </c>
+      <c r="C442" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="D442" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E442" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F442" s="3" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="443" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A443" s="4">
+        <v>442</v>
+      </c>
+      <c r="B443" s="5" t="s">
+        <v>953</v>
+      </c>
+      <c r="C443" s="5" t="s">
+        <v>954</v>
+      </c>
+      <c r="D443" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E443" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F443" s="5" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="444" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A444" s="2">
+        <v>443</v>
+      </c>
+      <c r="B444" s="3" t="s">
+        <v>956</v>
+      </c>
+      <c r="C444" s="3" t="s">
+        <v>954</v>
+      </c>
+      <c r="D444" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E444" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F444" s="3" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="445" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A445" s="4">
+        <v>444</v>
+      </c>
+      <c r="B445" s="5" t="s">
+        <v>958</v>
+      </c>
+      <c r="C445" s="5" t="s">
+        <v>954</v>
+      </c>
+      <c r="D445" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E445" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F445" s="5" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="446" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A446" s="2">
+        <v>445</v>
+      </c>
+      <c r="B446" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="C446" s="3" t="s">
+        <v>954</v>
+      </c>
+      <c r="D446" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E446" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F446" s="3" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="447" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A447" s="4">
+        <v>446</v>
+      </c>
+      <c r="B447" s="5" t="s">
+        <v>962</v>
+      </c>
+      <c r="C447" s="5" t="s">
+        <v>954</v>
+      </c>
+      <c r="D447" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E447" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F447" s="5" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="448" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A448" s="2">
+        <v>447</v>
+      </c>
+      <c r="B448" s="3" t="s">
+        <v>964</v>
+      </c>
+      <c r="C448" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D448" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E448" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F448" s="3" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="449" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A449" s="4">
+        <v>448</v>
+      </c>
+      <c r="B449" s="5" t="s">
+        <v>966</v>
+      </c>
+      <c r="C449" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D449" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E449" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F449" s="5" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="450" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A450" s="2">
+        <v>449</v>
+      </c>
+      <c r="B450" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="C450" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D450" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E450" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F450" s="3" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="451" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A451" s="4">
+        <v>450</v>
+      </c>
+      <c r="B451" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="C451" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D451" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E451" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F451" s="5" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="452" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A452" s="2">
+        <v>451</v>
+      </c>
+      <c r="B452" s="3" t="s">
+        <v>972</v>
+      </c>
+      <c r="C452" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="D452" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E452" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F452" s="3" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="453" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A453" s="4">
+        <v>452</v>
+      </c>
+      <c r="B453" s="5" t="s">
+        <v>974</v>
+      </c>
+      <c r="C453" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="D453" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E453" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F453" s="5" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="454" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A454" s="2">
+        <v>453</v>
+      </c>
+      <c r="B454" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="C454" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="D454" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E454" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F454" s="3" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="455" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A455" s="4">
+        <v>454</v>
+      </c>
+      <c r="B455" s="5" t="s">
+        <v>978</v>
+      </c>
+      <c r="C455" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="D455" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E455" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F455" s="5" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="456" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A456" s="2">
+        <v>455</v>
+      </c>
+      <c r="B456" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="C456" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D456" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E456" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F456" s="3" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="457" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A457" s="4">
+        <v>456</v>
+      </c>
+      <c r="B457" s="5" t="s">
+        <v>982</v>
+      </c>
+      <c r="C457" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D457" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E457" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F457" s="5" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="458" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A458" s="2">
+        <v>457</v>
+      </c>
+      <c r="B458" s="3" t="s">
+        <v>984</v>
+      </c>
+      <c r="C458" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D458" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E458" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F458" s="3" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="459" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A459" s="4">
+        <v>458</v>
+      </c>
+      <c r="B459" s="5" t="s">
+        <v>986</v>
+      </c>
+      <c r="C459" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D459" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E459" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F459" s="5" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="460" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A460" s="2">
+        <v>459</v>
+      </c>
+      <c r="B460" s="3" t="s">
+        <v>988</v>
+      </c>
+      <c r="C460" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D460" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E460" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F460" s="3" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="461" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A461" s="4">
+        <v>460</v>
+      </c>
+      <c r="B461" s="5" t="s">
+        <v>990</v>
+      </c>
+      <c r="C461" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D461" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E461" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F461" s="5" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="462" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A462" s="2">
+        <v>461</v>
+      </c>
+      <c r="B462" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="C462" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="D462" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E462" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F462" s="3" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="463" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A463" s="4">
+        <v>462</v>
+      </c>
+      <c r="B463" s="5" t="s">
+        <v>994</v>
+      </c>
+      <c r="C463" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D463" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E463" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F463" s="5" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="464" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A464" s="2">
+        <v>463</v>
+      </c>
+      <c r="B464" s="3" t="s">
+        <v>996</v>
+      </c>
+      <c r="C464" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D464" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E464" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F464" s="3" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="465" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A465" s="4">
+        <v>464</v>
+      </c>
+      <c r="B465" s="5" t="s">
+        <v>998</v>
+      </c>
+      <c r="C465" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D465" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E465" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F465" s="5" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="466" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A466" s="2">
+        <v>465</v>
+      </c>
+      <c r="B466" s="3" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C466" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="D466" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E466" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F466" s="3" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="467" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A467" s="4">
+        <v>466</v>
+      </c>
+      <c r="B467" s="5" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C467" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D467" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E467" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F467" s="5" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="468" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A468" s="2">
+        <v>467</v>
+      </c>
+      <c r="B468" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="C468" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D468" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E468" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F468" s="3" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="469" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A469" s="4">
+        <v>468</v>
+      </c>
+      <c r="B469" s="5" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C469" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D469" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E469" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F469" s="5" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="470" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A470" s="2">
+        <v>469</v>
+      </c>
+      <c r="B470" s="3" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C470" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D470" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E470" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F470" s="3" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="471" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A471" s="4">
+        <v>470</v>
+      </c>
+      <c r="B471" s="5" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C471" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="D471" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E471" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F471" s="5" t="s">
+        <v>1011</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Update pipelines with standardized credential variables
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="1012">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="1017">
   <si>
     <t>Run #</t>
   </si>
@@ -3047,6 +3047,21 @@
   </si>
   <si>
     <t>03/06/2026, 21:38:34</t>
+  </si>
+  <si>
+    <t>CP-MLI-084099155</t>
+  </si>
+  <si>
+    <t>TC_SAN_002 | Create Commercial England &amp; Wales policy (multiple products) via referral</t>
+  </si>
+  <si>
+    <t>04/06/2026, 16:51:50</t>
+  </si>
+  <si>
+    <t>CP-MLI-084100155</t>
+  </si>
+  <si>
+    <t>04/06/2026, 16:54:06</t>
   </si>
 </sst>
 </file>
@@ -3480,7 +3495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F471"/>
+  <dimension ref="A1:F473"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -12911,6 +12926,46 @@
         <v>1011</v>
       </c>
     </row>
+    <row r="472" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A472" s="2">
+        <v>471</v>
+      </c>
+      <c r="B472" s="3" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C472" s="3" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D472" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E472" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F472" s="3" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="473" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A473" s="4">
+        <v>472</v>
+      </c>
+      <c r="B473" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C473" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D473" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E473" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F473" s="5" t="s">
+        <v>1016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
updated branch with latest changes
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2371" uniqueCount="1020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2666" uniqueCount="1146">
   <si>
     <t>Run #</t>
   </si>
@@ -3071,6 +3071,384 @@
   </si>
   <si>
     <t>23/06/2026, 17:11:06</t>
+  </si>
+  <si>
+    <t>CP-NI-058372175</t>
+  </si>
+  <si>
+    <t>TC_BDX_001 | Commercial quote with Address line 1-4 and City at 255 chars, NB policy, CNR, MTA future date premium 300, cancel only MTA</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:22:32</t>
+  </si>
+  <si>
+    <t>DA-MLI-058374175</t>
+  </si>
+  <si>
+    <t>TC_BDX_002_INTER_COMM | Create Residential NB policy, MTA1/MTA2, CNR_MTA and cancel from inception with BDX lines</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:32:12</t>
+  </si>
+  <si>
+    <t>DA-MLI-058376175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:37:04</t>
+  </si>
+  <si>
+    <t>DA-MLI-058377175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:38:46</t>
+  </si>
+  <si>
+    <t>DA-MLI-058381175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:44:56</t>
+  </si>
+  <si>
+    <t>DA-MLI-058385175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 20:52:03</t>
+  </si>
+  <si>
+    <t>DA-MLI-058389175</t>
+  </si>
+  <si>
+    <t>TC_BDX_003_BDE_COMM | Create Residential NB policy, MTA (350.67), CNR with reason and verify BDX lines</t>
+  </si>
+  <si>
+    <t>24/06/2026, 21:00:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-058390175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 21:03:03</t>
+  </si>
+  <si>
+    <t>DA-MLI-058393175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 21:09:07</t>
+  </si>
+  <si>
+    <t>CP-NI-058397175</t>
+  </si>
+  <si>
+    <t>24/06/2026, 21:17:30</t>
+  </si>
+  <si>
+    <t>CP-MLI-058400175</t>
+  </si>
+  <si>
+    <t>TC_BDX_001 | England &amp; Wales Commercial quote with Address line 1-4 and City at 255 chars, NB policy, CNR, MTA future date premium 300, cancel only MTA</t>
+  </si>
+  <si>
+    <t>24/06/2026, 22:06:32</t>
+  </si>
+  <si>
+    <t>CP-MLI-058412176</t>
+  </si>
+  <si>
+    <t>TC_BDX_001 | England &amp; Wales Commercial NB policy, CNR, MTA future date premium 300, cancel only MTA</t>
+  </si>
+  <si>
+    <t>25/06/2026, 11:32:14</t>
+  </si>
+  <si>
+    <t>CP-MLI-058414176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 11:36:52</t>
+  </si>
+  <si>
+    <t>DA-MLI-058419176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 12:10:23</t>
+  </si>
+  <si>
+    <t>DA-MLI-058423176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 12:17:55</t>
+  </si>
+  <si>
+    <t>CP-MLI-058430176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 14:31:42</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058467176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 18:48:35</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058472176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 18:50:18</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058475176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 18:56:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-058559176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 20:48:29</t>
+  </si>
+  <si>
+    <t>DA-MLI-058563176</t>
+  </si>
+  <si>
+    <t>25/06/2026, 20:54:30</t>
+  </si>
+  <si>
+    <t>DA-MLI-058731177</t>
+  </si>
+  <si>
+    <t>26/06/2026, 15:23:41</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058755177</t>
+  </si>
+  <si>
+    <t>26/06/2026, 18:09:59</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058915180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 10:46:59</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058918180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 10:57:51</t>
+  </si>
+  <si>
+    <t>DA-MLI-058938180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:10:33</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058940180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:15:09</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-058943180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:19:48</t>
+  </si>
+  <si>
+    <t>CP-MLI-058946180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:42:54</t>
+  </si>
+  <si>
+    <t>CP-MLI-058948180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:44:32</t>
+  </si>
+  <si>
+    <t>CP-MLI-058949180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 14:46:46</t>
+  </si>
+  <si>
+    <t>CP-MLI-058954180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 15:04:45</t>
+  </si>
+  <si>
+    <t>CP-MLI-058961180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 15:20:47</t>
+  </si>
+  <si>
+    <t>CP-MLI-058964180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 15:25:45</t>
+  </si>
+  <si>
+    <t>CP-MLI-086636180</t>
+  </si>
+  <si>
+    <t>29/06/2026, 15:46:02</t>
+  </si>
+  <si>
+    <t>DA-MLI-541203181</t>
+  </si>
+  <si>
+    <t>30/06/2026, 15:43:23</t>
+  </si>
+  <si>
+    <t>DA-MLI-059158183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 08:39:15</t>
+  </si>
+  <si>
+    <t>DA-MLI-059161183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 08:43:50</t>
+  </si>
+  <si>
+    <t>DA-MLI-059168183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 08:59:17</t>
+  </si>
+  <si>
+    <t>CP-MLI-059175183</t>
+  </si>
+  <si>
+    <t>TC_SAN_020 | Trigger referral when limit exceeds 5M and product is Contaminated Land failed/further action search</t>
+  </si>
+  <si>
+    <t>02/07/2026, 11:47:43</t>
+  </si>
+  <si>
+    <t>DA-MLI-059198183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 13:26:55</t>
+  </si>
+  <si>
+    <t>DA-MLI-059199183</t>
+  </si>
+  <si>
+    <t>TC_REG_025 | Validate DA0045 Cancellation Notes field in BDX cancellation line</t>
+  </si>
+  <si>
+    <t>02/07/2026, 13:29:00</t>
+  </si>
+  <si>
+    <t>DA-MLI-059203183</t>
+  </si>
+  <si>
+    <t>TC_REG_026 | Verify DUAL Share GWP and BDX values through full cancellation flow</t>
+  </si>
+  <si>
+    <t>02/07/2026, 13:47:16</t>
+  </si>
+  <si>
+    <t>DA-MLI-059204183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:00:53</t>
+  </si>
+  <si>
+    <t>DA-MLI-059208183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:06:41</t>
+  </si>
+  <si>
+    <t>DA-MLI-059215183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:14:07</t>
+  </si>
+  <si>
+    <t>DA-MLI-059218183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:18:08</t>
+  </si>
+  <si>
+    <t>DA-MLI-059222183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:24:55</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-059224183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:29:42</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-059227183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:34:49</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-059229183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 14:36:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-059292183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:29:27</t>
+  </si>
+  <si>
+    <t>DA-MLI-059298183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:35:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-059304183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:41:21</t>
+  </si>
+  <si>
+    <t>DA-MLI-059305183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:43:01</t>
+  </si>
+  <si>
+    <t>DA-MLI-059308183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:47:13</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-059315183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 19:56:30</t>
+  </si>
+  <si>
+    <t>CP-MLI-PIE-059320183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 20:01:09</t>
+  </si>
+  <si>
+    <t>DA-MLI-086840183</t>
+  </si>
+  <si>
+    <t>02/07/2026, 20:14:12</t>
   </si>
 </sst>
 </file>
@@ -3504,7 +3882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F474"/>
+  <dimension ref="A1:F533"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -12995,6 +13373,1186 @@
         <v>1019</v>
       </c>
     </row>
+    <row r="475" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A475" s="4">
+        <v>474</v>
+      </c>
+      <c r="B475" s="5" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C475" s="5" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D475" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E475" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F475" s="5" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="476" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A476" s="2">
+        <v>475</v>
+      </c>
+      <c r="B476" s="3" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C476" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D476" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E476" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F476" s="3" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="477" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A477" s="4">
+        <v>476</v>
+      </c>
+      <c r="B477" s="5" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C477" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D477" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E477" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F477" s="5" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A478" s="2">
+        <v>477</v>
+      </c>
+      <c r="B478" s="3" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C478" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D478" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E478" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F478" s="3" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A479" s="4">
+        <v>478</v>
+      </c>
+      <c r="B479" s="5" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C479" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D479" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E479" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F479" s="5" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="480" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A480" s="2">
+        <v>479</v>
+      </c>
+      <c r="B480" s="3" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C480" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D480" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E480" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F480" s="3" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="481" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A481" s="4">
+        <v>480</v>
+      </c>
+      <c r="B481" s="5" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C481" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D481" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E481" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F481" s="5" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="482" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A482" s="2">
+        <v>481</v>
+      </c>
+      <c r="B482" s="3" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C482" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D482" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E482" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F482" s="3" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="483" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A483" s="4">
+        <v>482</v>
+      </c>
+      <c r="B483" s="5" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C483" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D483" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E483" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F483" s="5" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="484" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A484" s="2">
+        <v>483</v>
+      </c>
+      <c r="B484" s="3" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C484" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D484" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E484" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F484" s="3" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="485" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A485" s="4">
+        <v>484</v>
+      </c>
+      <c r="B485" s="5" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C485" s="5" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D485" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E485" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F485" s="5" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="486" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A486" s="2">
+        <v>485</v>
+      </c>
+      <c r="B486" s="3" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C486" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D486" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E486" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F486" s="3" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="487" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A487" s="4">
+        <v>486</v>
+      </c>
+      <c r="B487" s="5" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C487" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D487" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E487" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F487" s="5" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="488" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A488" s="2">
+        <v>487</v>
+      </c>
+      <c r="B488" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C488" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D488" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E488" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F488" s="3" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="489" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A489" s="4">
+        <v>488</v>
+      </c>
+      <c r="B489" s="5" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C489" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D489" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E489" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F489" s="5" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="490" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A490" s="2">
+        <v>489</v>
+      </c>
+      <c r="B490" s="3" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C490" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D490" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E490" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F490" s="3" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="491" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A491" s="4">
+        <v>490</v>
+      </c>
+      <c r="B491" s="5" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C491" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D491" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E491" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F491" s="5" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="492" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A492" s="2">
+        <v>491</v>
+      </c>
+      <c r="B492" s="3" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C492" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D492" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E492" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F492" s="3" t="s">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="493" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A493" s="4">
+        <v>492</v>
+      </c>
+      <c r="B493" s="5" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C493" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D493" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E493" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F493" s="5" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="494" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A494" s="2">
+        <v>493</v>
+      </c>
+      <c r="B494" s="3" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C494" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D494" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E494" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F494" s="3" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="495" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A495" s="4">
+        <v>494</v>
+      </c>
+      <c r="B495" s="5" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C495" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D495" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E495" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F495" s="5" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="496" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A496" s="2">
+        <v>495</v>
+      </c>
+      <c r="B496" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C496" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="D496" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E496" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F496" s="3" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="497" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A497" s="4">
+        <v>496</v>
+      </c>
+      <c r="B497" s="5" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C497" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D497" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E497" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F497" s="5" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="498" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A498" s="2">
+        <v>497</v>
+      </c>
+      <c r="B498" s="3" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C498" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D498" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E498" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F498" s="3" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="499" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A499" s="4">
+        <v>498</v>
+      </c>
+      <c r="B499" s="5" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C499" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D499" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E499" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F499" s="5" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="500" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A500" s="2">
+        <v>499</v>
+      </c>
+      <c r="B500" s="3" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C500" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="D500" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E500" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F500" s="3" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="501" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A501" s="4">
+        <v>500</v>
+      </c>
+      <c r="B501" s="5" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C501" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D501" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E501" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F501" s="5" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="502" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A502" s="2">
+        <v>501</v>
+      </c>
+      <c r="B502" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C502" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D502" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E502" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F502" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="503" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A503" s="4">
+        <v>502</v>
+      </c>
+      <c r="B503" s="5" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C503" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D503" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E503" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F503" s="5" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="504" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A504" s="2">
+        <v>503</v>
+      </c>
+      <c r="B504" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C504" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D504" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E504" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F504" s="3" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="505" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A505" s="4">
+        <v>504</v>
+      </c>
+      <c r="B505" s="5" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C505" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D505" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E505" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F505" s="5" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="506" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A506" s="2">
+        <v>505</v>
+      </c>
+      <c r="B506" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C506" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D506" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E506" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F506" s="3" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="507" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A507" s="4">
+        <v>506</v>
+      </c>
+      <c r="B507" s="5" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C507" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D507" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E507" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F507" s="5" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="508" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A508" s="2">
+        <v>507</v>
+      </c>
+      <c r="B508" s="3" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C508" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D508" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E508" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F508" s="3" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="509" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A509" s="4">
+        <v>508</v>
+      </c>
+      <c r="B509" s="5" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C509" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D509" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E509" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F509" s="5" t="s">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="510" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A510" s="2">
+        <v>509</v>
+      </c>
+      <c r="B510" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C510" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D510" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E510" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="F510" s="3" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="511" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A511" s="4">
+        <v>510</v>
+      </c>
+      <c r="B511" s="5" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C511" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D511" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E511" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F511" s="5" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="512" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A512" s="2">
+        <v>511</v>
+      </c>
+      <c r="B512" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C512" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D512" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E512" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F512" s="3" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="513" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A513" s="4">
+        <v>512</v>
+      </c>
+      <c r="B513" s="5" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C513" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D513" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E513" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F513" s="5" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="514" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A514" s="2">
+        <v>513</v>
+      </c>
+      <c r="B514" s="3" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C514" s="3" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D514" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E514" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F514" s="3" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="515" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A515" s="4">
+        <v>514</v>
+      </c>
+      <c r="B515" s="5" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C515" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="D515" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E515" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F515" s="5" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="516" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A516" s="2">
+        <v>515</v>
+      </c>
+      <c r="B516" s="3" t="s">
+        <v>1108</v>
+      </c>
+      <c r="C516" s="3" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D516" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E516" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F516" s="3" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="517" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A517" s="4">
+        <v>516</v>
+      </c>
+      <c r="B517" s="5" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C517" s="5" t="s">
+        <v>1112</v>
+      </c>
+      <c r="D517" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E517" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F517" s="5" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="518" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A518" s="2">
+        <v>517</v>
+      </c>
+      <c r="B518" s="3" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C518" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D518" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E518" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F518" s="3" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="519" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A519" s="4">
+        <v>518</v>
+      </c>
+      <c r="B519" s="5" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C519" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D519" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E519" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F519" s="5" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="520" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A520" s="2">
+        <v>519</v>
+      </c>
+      <c r="B520" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C520" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D520" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E520" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F520" s="3" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="521" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A521" s="4">
+        <v>520</v>
+      </c>
+      <c r="B521" s="5" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C521" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D521" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E521" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F521" s="5" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="522" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A522" s="2">
+        <v>521</v>
+      </c>
+      <c r="B522" s="3" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C522" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D522" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E522" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F522" s="3" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="523" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A523" s="4">
+        <v>522</v>
+      </c>
+      <c r="B523" s="5" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C523" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D523" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E523" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F523" s="5" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="524" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A524" s="2">
+        <v>523</v>
+      </c>
+      <c r="B524" s="3" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C524" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D524" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E524" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F524" s="3" t="s">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="525" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A525" s="4">
+        <v>524</v>
+      </c>
+      <c r="B525" s="5" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C525" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D525" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E525" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F525" s="5" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="526" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A526" s="2">
+        <v>525</v>
+      </c>
+      <c r="B526" s="3" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C526" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D526" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E526" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F526" s="3" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="527" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A527" s="4">
+        <v>526</v>
+      </c>
+      <c r="B527" s="5" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C527" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D527" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E527" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F527" s="5" t="s">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="528" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A528" s="2">
+        <v>527</v>
+      </c>
+      <c r="B528" s="3" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C528" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D528" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E528" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F528" s="3" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="529" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A529" s="4">
+        <v>528</v>
+      </c>
+      <c r="B529" s="5" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C529" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D529" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E529" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F529" s="5" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="530" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A530" s="2">
+        <v>529</v>
+      </c>
+      <c r="B530" s="3" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C530" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D530" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E530" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F530" s="3" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="531" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A531" s="4">
+        <v>530</v>
+      </c>
+      <c r="B531" s="5" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C531" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D531" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E531" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F531" s="5" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="532" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A532" s="2">
+        <v>531</v>
+      </c>
+      <c r="B532" s="3" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C532" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D532" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E532" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F532" s="3" t="s">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="533" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A533" s="4">
+        <v>532</v>
+      </c>
+      <c r="B533" s="5" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C533" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D533" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E533" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F533" s="5" t="s">
+        <v>1145</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
chore: sync local framework updates
</commit_message>
<xml_diff>
--- a/reports/policy-tracker.xlsx
+++ b/reports/policy-tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2811" uniqueCount="1206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2851" uniqueCount="1223">
   <si>
     <t>Run #</t>
   </si>
@@ -3629,6 +3629,57 @@
   </si>
   <si>
     <t>09/07/2026, 19:04:56</t>
+  </si>
+  <si>
+    <t>CP-NI-061751191</t>
+  </si>
+  <si>
+    <t>TC_REG_057 | NB Clauses are correctly generated .</t>
+  </si>
+  <si>
+    <t>10/07/2026, 15:43:16</t>
+  </si>
+  <si>
+    <t>CP-NI-061752191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 15:50:24</t>
+  </si>
+  <si>
+    <t>CP-NI-061753191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 15:59:03</t>
+  </si>
+  <si>
+    <t>CP-NI-061754191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 16:02:23</t>
+  </si>
+  <si>
+    <t>CP-NI-061755191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 16:05:02</t>
+  </si>
+  <si>
+    <t>CP-NI-061756191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 16:11:49</t>
+  </si>
+  <si>
+    <t>CP-NI-061757191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 16:14:08</t>
+  </si>
+  <si>
+    <t>CP-NI-061763191</t>
+  </si>
+  <si>
+    <t>10/07/2026, 16:28:19</t>
   </si>
 </sst>
 </file>
@@ -4062,7 +4113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F562"/>
+  <dimension ref="A1:F570"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -15313,6 +15364,166 @@
         <v>1205</v>
       </c>
     </row>
+    <row r="563" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A563" s="4">
+        <v>562</v>
+      </c>
+      <c r="B563" s="5" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C563" s="5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D563" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E563" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F563" s="5" t="s">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="564" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A564" s="2">
+        <v>563</v>
+      </c>
+      <c r="B564" s="3" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C564" s="3" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D564" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E564" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F564" s="3" t="s">
+        <v>1210</v>
+      </c>
+    </row>
+    <row r="565" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A565" s="4">
+        <v>564</v>
+      </c>
+      <c r="B565" s="5" t="s">
+        <v>1211</v>
+      </c>
+      <c r="C565" s="5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D565" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E565" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F565" s="5" t="s">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="566" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A566" s="2">
+        <v>565</v>
+      </c>
+      <c r="B566" s="3" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C566" s="3" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D566" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E566" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F566" s="3" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="567" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A567" s="4">
+        <v>566</v>
+      </c>
+      <c r="B567" s="5" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C567" s="5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D567" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E567" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F567" s="5" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="568" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A568" s="2">
+        <v>567</v>
+      </c>
+      <c r="B568" s="3" t="s">
+        <v>1217</v>
+      </c>
+      <c r="C568" s="3" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D568" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E568" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F568" s="3" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="569" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A569" s="4">
+        <v>568</v>
+      </c>
+      <c r="B569" s="5" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C569" s="5" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D569" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E569" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="F569" s="5" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="570" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A570" s="2">
+        <v>569</v>
+      </c>
+      <c r="B570" s="3" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C570" s="3" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D570" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E570" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="F570" s="3" t="s">
+        <v>1222</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>